<commit_message>
Application Attribute Testing: list all references per attribute
Each attribute section now shows every evidence reference behind that
attribute (from the original attribute testing) to the right of the
section, one clickable cell per ref (columns H onward) that opens its
evidence review entry; key evidence is highlighted green. Contents shows
the key refs and the total number of references per section.
268 links verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VJjJPWjXw5ntc2ii5NsFQ1
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION.xlsx
+++ b/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION.xlsx
@@ -356,7 +356,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -516,11 +516,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -729,6 +743,15 @@
     </xf>
     <xf numFmtId="0" fontId="36" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="20" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5512,7 +5535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G167"/>
+  <dimension ref="A1:AA167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="8.75" customWidth="1" style="73" min="1" max="1"/>
@@ -5522,6 +5545,35 @@
     <col width="61.5" customWidth="1" style="73" min="5" max="5"/>
     <col width="113.75" customWidth="1" style="73" min="6" max="6"/>
     <col width="48.08203125" customWidth="1" style="73" min="7" max="7"/>
+    <col width="8" customWidth="1" style="73" min="8" max="8"/>
+    <col width="8" customWidth="1" style="73" min="9" max="9"/>
+    <col width="8" customWidth="1" style="73" min="10" max="10"/>
+    <col width="8" customWidth="1" style="73" min="11" max="11"/>
+    <col width="8" customWidth="1" style="73" min="12" max="12"/>
+    <col width="8" customWidth="1" style="73" min="13" max="13"/>
+    <col width="8" customWidth="1" style="73" min="14" max="14"/>
+    <col width="8" customWidth="1" style="73" min="15" max="15"/>
+    <col width="8" customWidth="1" style="73" min="16" max="16"/>
+    <col width="8" customWidth="1" style="73" min="17" max="17"/>
+    <col width="8" customWidth="1" style="73" min="18" max="18"/>
+    <col width="8" customWidth="1" style="73" min="19" max="19"/>
+    <col width="8" customWidth="1" style="73" min="20" max="20"/>
+    <col width="8" customWidth="1" style="73" min="21" max="21"/>
+    <col width="8" customWidth="1" style="73" min="22" max="22"/>
+    <col width="8" customWidth="1" style="73" min="23" max="23"/>
+    <col width="8" customWidth="1" style="73" min="24" max="24"/>
+    <col width="8" customWidth="1" style="73" min="25" max="25"/>
+    <col width="8" customWidth="1" style="73" min="26" max="26"/>
+    <col width="8" customWidth="1" style="73" min="27" max="27"/>
+    <col width="8" customWidth="1" style="73" min="28" max="28"/>
+    <col width="8" customWidth="1" style="73" min="29" max="29"/>
+    <col width="8" customWidth="1" style="73" min="30" max="30"/>
+    <col width="8" customWidth="1" style="73" min="31" max="31"/>
+    <col width="8" customWidth="1" style="73" min="32" max="32"/>
+    <col width="8" customWidth="1" style="73" min="33" max="33"/>
+    <col width="8" customWidth="1" style="73" min="34" max="34"/>
+    <col width="8" customWidth="1" style="73" min="35" max="35"/>
+    <col width="8" customWidth="1" style="73" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.5" customHeight="1" s="73">
@@ -5576,7 +5628,7 @@
       </c>
       <c r="D3" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – MA01</t>
+          <t>Key: MA01 · 6 references in total</t>
         </is>
       </c>
       <c r="E3" s="66" t="n"/>
@@ -5605,7 +5657,7 @@
       </c>
       <c r="D4" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E01</t>
+          <t>Key: E01 · 9 references in total</t>
         </is>
       </c>
       <c r="E4" s="66" t="n"/>
@@ -5663,7 +5715,7 @@
       </c>
       <c r="D6" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E03</t>
+          <t>Key: E03 · 9 references in total</t>
         </is>
       </c>
       <c r="E6" s="66" t="n"/>
@@ -5692,7 +5744,7 @@
       </c>
       <c r="D7" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E03</t>
+          <t>Key: E03 · 10 references in total</t>
         </is>
       </c>
       <c r="E7" s="66" t="n"/>
@@ -5721,7 +5773,7 @@
       </c>
       <c r="D8" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E03</t>
+          <t>Key: E03 · 16 references in total</t>
         </is>
       </c>
       <c r="E8" s="66" t="n"/>
@@ -5750,7 +5802,7 @@
       </c>
       <c r="D9" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E03</t>
+          <t>Key: E03 · 16 references in total</t>
         </is>
       </c>
       <c r="E9" s="66" t="n"/>
@@ -5779,7 +5831,7 @@
       </c>
       <c r="D10" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E03</t>
+          <t>Key: E03 · 7 references in total</t>
         </is>
       </c>
       <c r="E10" s="66" t="n"/>
@@ -5808,7 +5860,7 @@
       </c>
       <c r="D11" s="65" t="inlineStr">
         <is>
-          <t>5 file(s) – BLA06, DMA01, DMA02, DMA03, DMA04</t>
+          <t>Key: BLA06, DMA01, DMA02, DMA03, DMA04 · 14 references in total</t>
         </is>
       </c>
       <c r="E11" s="66" t="n"/>
@@ -5837,7 +5889,7 @@
       </c>
       <c r="D12" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E03</t>
+          <t>Key: E03 · 6 references in total</t>
         </is>
       </c>
       <c r="E12" s="66" t="n"/>
@@ -5866,7 +5918,7 @@
       </c>
       <c r="D13" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E01</t>
+          <t>Key: E01 · 8 references in total</t>
         </is>
       </c>
       <c r="E13" s="66" t="n"/>
@@ -5895,7 +5947,7 @@
       </c>
       <c r="D14" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – E05</t>
+          <t>Key: E05 · 11 references in total</t>
         </is>
       </c>
       <c r="E14" s="66" t="n"/>
@@ -5924,7 +5976,7 @@
       </c>
       <c r="D15" s="65" t="inlineStr">
         <is>
-          <t>1 file(s) – MA01</t>
+          <t>Key: MA01 · 6 references in total</t>
         </is>
       </c>
       <c r="E15" s="66" t="n"/>
@@ -5953,7 +6005,7 @@
       </c>
       <c r="D16" s="65" t="inlineStr">
         <is>
-          <t>5 file(s) – BLA06, DMA01, DMA02, DMA03, DMA04</t>
+          <t>Key: BLA06, DMA01, DMA02, DMA03, DMA04 · 20 references in total</t>
         </is>
       </c>
       <c r="E16" s="66" t="n"/>
@@ -6093,6 +6145,11 @@
       <c r="G22" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H22" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (6) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -6152,6 +6209,36 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H23" s="90" t="inlineStr">
+        <is>
+          <t>MA01</t>
+        </is>
+      </c>
+      <c r="I23" s="91" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="J23" s="91" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="K23" s="91" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="L23" s="91" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="M23" s="91" t="inlineStr">
+        <is>
+          <t>E16b</t>
+        </is>
+      </c>
     </row>
     <row r="24" s="73"/>
     <row r="25" ht="15.5" customHeight="1" s="73">
@@ -6195,6 +6282,11 @@
       <c r="G26" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H26" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (9) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -6246,6 +6338,51 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H27" s="91" t="inlineStr">
+        <is>
+          <t>BLA01</t>
+        </is>
+      </c>
+      <c r="I27" s="91" t="inlineStr">
+        <is>
+          <t>BLA02</t>
+        </is>
+      </c>
+      <c r="J27" s="91" t="inlineStr">
+        <is>
+          <t>BLA03</t>
+        </is>
+      </c>
+      <c r="K27" s="91" t="inlineStr">
+        <is>
+          <t>BLA04</t>
+        </is>
+      </c>
+      <c r="L27" s="91" t="inlineStr">
+        <is>
+          <t>BLA05</t>
+        </is>
+      </c>
+      <c r="M27" s="91" t="inlineStr">
+        <is>
+          <t>DMA02</t>
+        </is>
+      </c>
+      <c r="N27" s="90" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="O27" s="91" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="P27" s="91" t="inlineStr">
+        <is>
+          <t>E16b</t>
+        </is>
+      </c>
     </row>
     <row r="28" s="73"/>
     <row r="29" s="73"/>
@@ -6290,6 +6427,11 @@
       <c r="G31" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H31" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (9) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -6340,6 +6482,51 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H32" s="91" t="inlineStr">
+        <is>
+          <t>BLA01</t>
+        </is>
+      </c>
+      <c r="I32" s="91" t="inlineStr">
+        <is>
+          <t>BLA02</t>
+        </is>
+      </c>
+      <c r="J32" s="91" t="inlineStr">
+        <is>
+          <t>BLA03</t>
+        </is>
+      </c>
+      <c r="K32" s="91" t="inlineStr">
+        <is>
+          <t>BLA04</t>
+        </is>
+      </c>
+      <c r="L32" s="91" t="inlineStr">
+        <is>
+          <t>BLA05</t>
+        </is>
+      </c>
+      <c r="M32" s="90" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="N32" s="91" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="O32" s="91" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
+      <c r="P32" s="91" t="inlineStr">
+        <is>
+          <t>E16b</t>
+        </is>
+      </c>
     </row>
     <row r="33" s="73"/>
     <row r="34" ht="15.5" customHeight="1" s="73">
@@ -6383,6 +6570,11 @@
       <c r="G35" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H35" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (10) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -6433,6 +6625,56 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H36" s="91" t="inlineStr">
+        <is>
+          <t>BLA01</t>
+        </is>
+      </c>
+      <c r="I36" s="91" t="inlineStr">
+        <is>
+          <t>BLA02</t>
+        </is>
+      </c>
+      <c r="J36" s="91" t="inlineStr">
+        <is>
+          <t>BLA03</t>
+        </is>
+      </c>
+      <c r="K36" s="91" t="inlineStr">
+        <is>
+          <t>BLA04</t>
+        </is>
+      </c>
+      <c r="L36" s="91" t="inlineStr">
+        <is>
+          <t>BLA05</t>
+        </is>
+      </c>
+      <c r="M36" s="90" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="N36" s="91" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="O36" s="91" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="P36" s="91" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="Q36" s="91" t="inlineStr">
+        <is>
+          <t>E16b</t>
+        </is>
+      </c>
     </row>
     <row r="37" s="73"/>
     <row r="38" ht="15.5" customHeight="1" s="73">
@@ -6476,6 +6718,11 @@
       <c r="G39" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H39" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (16) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -6526,6 +6773,86 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H40" s="91" t="inlineStr">
+        <is>
+          <t>BLA06</t>
+        </is>
+      </c>
+      <c r="I40" s="91" t="inlineStr">
+        <is>
+          <t>DMA01</t>
+        </is>
+      </c>
+      <c r="J40" s="91" t="inlineStr">
+        <is>
+          <t>DMA02</t>
+        </is>
+      </c>
+      <c r="K40" s="91" t="inlineStr">
+        <is>
+          <t>DMA03</t>
+        </is>
+      </c>
+      <c r="L40" s="91" t="inlineStr">
+        <is>
+          <t>DMA04</t>
+        </is>
+      </c>
+      <c r="M40" s="91" t="inlineStr">
+        <is>
+          <t>DMA05</t>
+        </is>
+      </c>
+      <c r="N40" s="91" t="inlineStr">
+        <is>
+          <t>DMA06</t>
+        </is>
+      </c>
+      <c r="O40" s="91" t="inlineStr">
+        <is>
+          <t>DMA07</t>
+        </is>
+      </c>
+      <c r="P40" s="91" t="inlineStr">
+        <is>
+          <t>DMA08</t>
+        </is>
+      </c>
+      <c r="Q40" s="91" t="inlineStr">
+        <is>
+          <t>DMA09</t>
+        </is>
+      </c>
+      <c r="R40" s="91" t="inlineStr">
+        <is>
+          <t>DMA10</t>
+        </is>
+      </c>
+      <c r="S40" s="91" t="inlineStr">
+        <is>
+          <t>DMA11</t>
+        </is>
+      </c>
+      <c r="T40" s="91" t="inlineStr">
+        <is>
+          <t>DMA12</t>
+        </is>
+      </c>
+      <c r="U40" s="90" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="V40" s="91" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="W40" s="91" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
     </row>
     <row r="41" s="73"/>
     <row r="42" ht="15.5" customHeight="1" s="73">
@@ -6569,6 +6896,11 @@
       <c r="G43" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H43" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (16) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -6619,6 +6951,86 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H44" s="91" t="inlineStr">
+        <is>
+          <t>BLA06</t>
+        </is>
+      </c>
+      <c r="I44" s="91" t="inlineStr">
+        <is>
+          <t>DMA01</t>
+        </is>
+      </c>
+      <c r="J44" s="91" t="inlineStr">
+        <is>
+          <t>DMA02</t>
+        </is>
+      </c>
+      <c r="K44" s="91" t="inlineStr">
+        <is>
+          <t>DMA03</t>
+        </is>
+      </c>
+      <c r="L44" s="91" t="inlineStr">
+        <is>
+          <t>DMA04</t>
+        </is>
+      </c>
+      <c r="M44" s="91" t="inlineStr">
+        <is>
+          <t>DMA05</t>
+        </is>
+      </c>
+      <c r="N44" s="91" t="inlineStr">
+        <is>
+          <t>DMA06</t>
+        </is>
+      </c>
+      <c r="O44" s="91" t="inlineStr">
+        <is>
+          <t>DMA07</t>
+        </is>
+      </c>
+      <c r="P44" s="91" t="inlineStr">
+        <is>
+          <t>DMA08</t>
+        </is>
+      </c>
+      <c r="Q44" s="91" t="inlineStr">
+        <is>
+          <t>DMA09</t>
+        </is>
+      </c>
+      <c r="R44" s="91" t="inlineStr">
+        <is>
+          <t>DMA10</t>
+        </is>
+      </c>
+      <c r="S44" s="91" t="inlineStr">
+        <is>
+          <t>DMA11</t>
+        </is>
+      </c>
+      <c r="T44" s="91" t="inlineStr">
+        <is>
+          <t>DMA12</t>
+        </is>
+      </c>
+      <c r="U44" s="90" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="V44" s="91" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="W44" s="91" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
     </row>
     <row r="45" s="73"/>
     <row r="46" ht="15.5" customHeight="1" s="73">
@@ -6662,6 +7074,11 @@
       <c r="G47" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H47" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (7) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -6712,6 +7129,41 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H48" s="91" t="inlineStr">
+        <is>
+          <t>BLA01</t>
+        </is>
+      </c>
+      <c r="I48" s="91" t="inlineStr">
+        <is>
+          <t>BLA02</t>
+        </is>
+      </c>
+      <c r="J48" s="91" t="inlineStr">
+        <is>
+          <t>BLA03</t>
+        </is>
+      </c>
+      <c r="K48" s="91" t="inlineStr">
+        <is>
+          <t>BLA04</t>
+        </is>
+      </c>
+      <c r="L48" s="91" t="inlineStr">
+        <is>
+          <t>BLA05</t>
+        </is>
+      </c>
+      <c r="M48" s="90" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="N48" s="91" t="inlineStr">
+        <is>
+          <t>E16b</t>
+        </is>
+      </c>
     </row>
     <row r="49" s="73"/>
     <row r="50" ht="15.5" customHeight="1" s="73">
@@ -6757,6 +7209,11 @@
           <t>Control Sample Assessment Result (Pass/Fail)</t>
         </is>
       </c>
+      <c r="H51" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (14) – click to open; key evidence in green</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="90" customHeight="1" s="73">
       <c r="A52" s="69" t="inlineStr">
@@ -6795,6 +7252,76 @@
       <c r="G52" s="67" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="H52" s="90" t="inlineStr">
+        <is>
+          <t>BLA06</t>
+        </is>
+      </c>
+      <c r="I52" s="90" t="inlineStr">
+        <is>
+          <t>DMA01</t>
+        </is>
+      </c>
+      <c r="J52" s="90" t="inlineStr">
+        <is>
+          <t>DMA02</t>
+        </is>
+      </c>
+      <c r="K52" s="90" t="inlineStr">
+        <is>
+          <t>DMA03</t>
+        </is>
+      </c>
+      <c r="L52" s="90" t="inlineStr">
+        <is>
+          <t>DMA04</t>
+        </is>
+      </c>
+      <c r="M52" s="91" t="inlineStr">
+        <is>
+          <t>DMA05</t>
+        </is>
+      </c>
+      <c r="N52" s="91" t="inlineStr">
+        <is>
+          <t>DMA06</t>
+        </is>
+      </c>
+      <c r="O52" s="91" t="inlineStr">
+        <is>
+          <t>DMA07</t>
+        </is>
+      </c>
+      <c r="P52" s="91" t="inlineStr">
+        <is>
+          <t>DMA08</t>
+        </is>
+      </c>
+      <c r="Q52" s="91" t="inlineStr">
+        <is>
+          <t>DMA09</t>
+        </is>
+      </c>
+      <c r="R52" s="91" t="inlineStr">
+        <is>
+          <t>DMA10</t>
+        </is>
+      </c>
+      <c r="S52" s="91" t="inlineStr">
+        <is>
+          <t>DMA11</t>
+        </is>
+      </c>
+      <c r="T52" s="91" t="inlineStr">
+        <is>
+          <t>DMA12</t>
+        </is>
+      </c>
+      <c r="U52" s="91" t="inlineStr">
+        <is>
+          <t>E09</t>
         </is>
       </c>
     </row>
@@ -7007,6 +7534,11 @@
       <c r="G59" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H59" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (6) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -7057,6 +7589,36 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H60" s="91" t="inlineStr">
+        <is>
+          <t>MA01</t>
+        </is>
+      </c>
+      <c r="I60" s="91" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="J60" s="91" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="K60" s="90" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="L60" s="91" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="M60" s="91" t="inlineStr">
+        <is>
+          <t>E16b</t>
+        </is>
+      </c>
     </row>
     <row r="61" s="73"/>
     <row r="62" ht="15.5" customHeight="1" s="73">
@@ -7100,6 +7662,11 @@
       <c r="G63" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H63" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (8) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -7151,6 +7718,46 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H64" s="91" t="inlineStr">
+        <is>
+          <t>BLA01</t>
+        </is>
+      </c>
+      <c r="I64" s="91" t="inlineStr">
+        <is>
+          <t>BLA02</t>
+        </is>
+      </c>
+      <c r="J64" s="91" t="inlineStr">
+        <is>
+          <t>BLA03</t>
+        </is>
+      </c>
+      <c r="K64" s="91" t="inlineStr">
+        <is>
+          <t>BLA04</t>
+        </is>
+      </c>
+      <c r="L64" s="91" t="inlineStr">
+        <is>
+          <t>BLA05</t>
+        </is>
+      </c>
+      <c r="M64" s="91" t="inlineStr">
+        <is>
+          <t>DMA02</t>
+        </is>
+      </c>
+      <c r="N64" s="90" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="O64" s="91" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
     </row>
     <row r="65" s="73"/>
     <row r="66" ht="15.5" customHeight="1" s="73">
@@ -7194,6 +7801,11 @@
       <c r="G67" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H67" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (11) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -7244,6 +7856,61 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H68" s="91" t="inlineStr">
+        <is>
+          <t>BLA01</t>
+        </is>
+      </c>
+      <c r="I68" s="91" t="inlineStr">
+        <is>
+          <t>BLA02</t>
+        </is>
+      </c>
+      <c r="J68" s="91" t="inlineStr">
+        <is>
+          <t>BLA03</t>
+        </is>
+      </c>
+      <c r="K68" s="91" t="inlineStr">
+        <is>
+          <t>BLA04</t>
+        </is>
+      </c>
+      <c r="L68" s="91" t="inlineStr">
+        <is>
+          <t>BLA05</t>
+        </is>
+      </c>
+      <c r="M68" s="91" t="inlineStr">
+        <is>
+          <t>DMA02</t>
+        </is>
+      </c>
+      <c r="N68" s="91" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="O68" s="90" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="P68" s="91" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="Q68" s="91" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
+      <c r="R68" s="91" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
     </row>
     <row r="69" s="73"/>
     <row r="70" ht="15.5" customHeight="1" s="73">
@@ -7287,6 +7954,11 @@
       <c r="G71" s="62" t="inlineStr">
         <is>
           <t>Control Sample Assessment Result (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="H71" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (6) – click to open; key evidence in green</t>
         </is>
       </c>
     </row>
@@ -7346,6 +8018,36 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="H72" s="91" t="inlineStr">
+        <is>
+          <t>DMA02</t>
+        </is>
+      </c>
+      <c r="I72" s="90" t="inlineStr">
+        <is>
+          <t>MA01</t>
+        </is>
+      </c>
+      <c r="J72" s="91" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="K72" s="91" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="L72" s="91" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="M72" s="91" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
     </row>
     <row r="73" s="73"/>
     <row r="74" ht="15.5" customHeight="1" s="73">
@@ -7391,6 +8093,11 @@
           <t>Control Sample Assessment Result (Pass/Fail)</t>
         </is>
       </c>
+      <c r="H75" s="89" t="inlineStr">
+        <is>
+          <t>All references for this attribute (20) – click to open; key evidence in green</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="78" customHeight="1" s="73">
       <c r="A76" s="69" t="inlineStr">
@@ -7429,6 +8136,106 @@
       <c r="G76" s="67" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="H76" s="91" t="inlineStr">
+        <is>
+          <t>BLA01</t>
+        </is>
+      </c>
+      <c r="I76" s="91" t="inlineStr">
+        <is>
+          <t>BLA02</t>
+        </is>
+      </c>
+      <c r="J76" s="91" t="inlineStr">
+        <is>
+          <t>BLA03</t>
+        </is>
+      </c>
+      <c r="K76" s="91" t="inlineStr">
+        <is>
+          <t>BLA04</t>
+        </is>
+      </c>
+      <c r="L76" s="91" t="inlineStr">
+        <is>
+          <t>BLA05</t>
+        </is>
+      </c>
+      <c r="M76" s="90" t="inlineStr">
+        <is>
+          <t>BLA06</t>
+        </is>
+      </c>
+      <c r="N76" s="90" t="inlineStr">
+        <is>
+          <t>DMA01</t>
+        </is>
+      </c>
+      <c r="O76" s="90" t="inlineStr">
+        <is>
+          <t>DMA02</t>
+        </is>
+      </c>
+      <c r="P76" s="90" t="inlineStr">
+        <is>
+          <t>DMA03</t>
+        </is>
+      </c>
+      <c r="Q76" s="90" t="inlineStr">
+        <is>
+          <t>DMA04</t>
+        </is>
+      </c>
+      <c r="R76" s="91" t="inlineStr">
+        <is>
+          <t>DMA05</t>
+        </is>
+      </c>
+      <c r="S76" s="91" t="inlineStr">
+        <is>
+          <t>DMA06</t>
+        </is>
+      </c>
+      <c r="T76" s="91" t="inlineStr">
+        <is>
+          <t>DMA07</t>
+        </is>
+      </c>
+      <c r="U76" s="91" t="inlineStr">
+        <is>
+          <t>DMA08</t>
+        </is>
+      </c>
+      <c r="V76" s="91" t="inlineStr">
+        <is>
+          <t>DMA09</t>
+        </is>
+      </c>
+      <c r="W76" s="91" t="inlineStr">
+        <is>
+          <t>DMA10</t>
+        </is>
+      </c>
+      <c r="X76" s="91" t="inlineStr">
+        <is>
+          <t>DMA11</t>
+        </is>
+      </c>
+      <c r="Y76" s="91" t="inlineStr">
+        <is>
+          <t>DMA12</t>
+        </is>
+      </c>
+      <c r="Z76" s="91" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="AA76" s="91" t="inlineStr">
+        <is>
+          <t>E09</t>
         </is>
       </c>
     </row>
@@ -10713,25 +11520,38 @@
     <row r="278" s="73"/>
     <row r="279" s="73"/>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="32">
+    <mergeCell ref="H59:M59"/>
+    <mergeCell ref="H47:N47"/>
     <mergeCell ref="A122:G122"/>
     <mergeCell ref="A91:G91"/>
+    <mergeCell ref="H67:R67"/>
     <mergeCell ref="A62:G62"/>
     <mergeCell ref="A156:G156"/>
     <mergeCell ref="A38:G38"/>
+    <mergeCell ref="H63:O63"/>
     <mergeCell ref="A58:G58"/>
     <mergeCell ref="A34:G34"/>
+    <mergeCell ref="H22:M22"/>
+    <mergeCell ref="H35:Q35"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A82:G82"/>
+    <mergeCell ref="H51:U51"/>
     <mergeCell ref="A107:G107"/>
+    <mergeCell ref="H43:W43"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H71:M71"/>
     <mergeCell ref="A70:G70"/>
+    <mergeCell ref="H39:W39"/>
     <mergeCell ref="A25:G25"/>
+    <mergeCell ref="H26:P26"/>
     <mergeCell ref="A46:G46"/>
     <mergeCell ref="A66:G66"/>
     <mergeCell ref="A74:G74"/>
+    <mergeCell ref="H75:AA75"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A50:G50"/>
+    <mergeCell ref="H31:P31"/>
     <mergeCell ref="A42:G42"/>
   </mergeCells>
   <hyperlinks>
@@ -10753,22 +11573,160 @@
     <hyperlink ref="B18" location="'Application Attribute Testing'!A122" display="Evidence reference table – evidence number → attribute tests"/>
     <hyperlink ref="B19" location="'Application Attribute Testing'!A156" display="Conclusion – all applications in scope (PASS) with evidence references"/>
     <hyperlink ref="A23" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink ref="H23" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink ref="I23" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink ref="J23" location="'Application Attribute Testing'!A111" display="E02"/>
+    <hyperlink ref="K23" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="L23" location="'Application Attribute Testing'!A113" display="E04"/>
+    <hyperlink ref="M23" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A27" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink ref="H27" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink ref="I27" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink ref="J27" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink ref="K27" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink ref="L27" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink ref="M27" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink ref="N27" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink ref="O27" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="P27" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A32" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="H32" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink ref="I32" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink ref="J32" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink ref="K32" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink ref="L32" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink ref="M32" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="N32" location="'Application Attribute Testing'!A113" display="E04"/>
+    <hyperlink ref="O32" location="'Application Attribute Testing'!A117" display="E09"/>
+    <hyperlink ref="P32" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A36" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="H36" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink ref="I36" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink ref="J36" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink ref="K36" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink ref="L36" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink ref="M36" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="N36" location="'Application Attribute Testing'!A113" display="E04"/>
+    <hyperlink ref="O36" location="'Application Attribute Testing'!A115" display="E07"/>
+    <hyperlink ref="P36" location="'Application Attribute Testing'!A116" display="E08"/>
+    <hyperlink ref="Q36" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A40" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="H40" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink ref="I40" location="'Application Attribute Testing'!A93" display="DMA01"/>
+    <hyperlink ref="J40" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink ref="K40" location="'Application Attribute Testing'!A95" display="DMA03"/>
+    <hyperlink ref="L40" location="'Application Attribute Testing'!A96" display="DMA04"/>
+    <hyperlink ref="M40" location="'Application Attribute Testing'!A97" display="DMA05"/>
+    <hyperlink ref="N40" location="'Application Attribute Testing'!A98" display="DMA06"/>
+    <hyperlink ref="O40" location="'Application Attribute Testing'!A99" display="DMA07"/>
+    <hyperlink ref="P40" location="'Application Attribute Testing'!A100" display="DMA08"/>
+    <hyperlink ref="Q40" location="'Application Attribute Testing'!A101" display="DMA09"/>
+    <hyperlink ref="R40" location="'Application Attribute Testing'!A102" display="DMA10"/>
+    <hyperlink ref="S40" location="'Application Attribute Testing'!A103" display="DMA11"/>
+    <hyperlink ref="T40" location="'Application Attribute Testing'!A104" display="DMA12"/>
+    <hyperlink ref="U40" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="V40" location="'Application Attribute Testing'!A113" display="E04"/>
+    <hyperlink ref="W40" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A44" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="H44" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink ref="I44" location="'Application Attribute Testing'!A93" display="DMA01"/>
+    <hyperlink ref="J44" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink ref="K44" location="'Application Attribute Testing'!A95" display="DMA03"/>
+    <hyperlink ref="L44" location="'Application Attribute Testing'!A96" display="DMA04"/>
+    <hyperlink ref="M44" location="'Application Attribute Testing'!A97" display="DMA05"/>
+    <hyperlink ref="N44" location="'Application Attribute Testing'!A98" display="DMA06"/>
+    <hyperlink ref="O44" location="'Application Attribute Testing'!A99" display="DMA07"/>
+    <hyperlink ref="P44" location="'Application Attribute Testing'!A100" display="DMA08"/>
+    <hyperlink ref="Q44" location="'Application Attribute Testing'!A101" display="DMA09"/>
+    <hyperlink ref="R44" location="'Application Attribute Testing'!A102" display="DMA10"/>
+    <hyperlink ref="S44" location="'Application Attribute Testing'!A103" display="DMA11"/>
+    <hyperlink ref="T44" location="'Application Attribute Testing'!A104" display="DMA12"/>
+    <hyperlink ref="U44" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="V44" location="'Application Attribute Testing'!A113" display="E04"/>
+    <hyperlink ref="W44" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A48" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="H48" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink ref="I48" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink ref="J48" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink ref="K48" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink ref="L48" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink ref="M48" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="N48" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A52" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink ref="H52" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink ref="I52" location="'Application Attribute Testing'!A93" display="DMA01"/>
+    <hyperlink ref="J52" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink ref="K52" location="'Application Attribute Testing'!A95" display="DMA03"/>
+    <hyperlink ref="L52" location="'Application Attribute Testing'!A96" display="DMA04"/>
+    <hyperlink ref="M52" location="'Application Attribute Testing'!A97" display="DMA05"/>
+    <hyperlink ref="N52" location="'Application Attribute Testing'!A98" display="DMA06"/>
+    <hyperlink ref="O52" location="'Application Attribute Testing'!A99" display="DMA07"/>
+    <hyperlink ref="P52" location="'Application Attribute Testing'!A100" display="DMA08"/>
+    <hyperlink ref="Q52" location="'Application Attribute Testing'!A101" display="DMA09"/>
+    <hyperlink ref="R52" location="'Application Attribute Testing'!A102" display="DMA10"/>
+    <hyperlink ref="S52" location="'Application Attribute Testing'!A103" display="DMA11"/>
+    <hyperlink ref="T52" location="'Application Attribute Testing'!A104" display="DMA12"/>
+    <hyperlink ref="U52" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A53" location="'Application Attribute Testing'!A93" display="DMA01"/>
     <hyperlink ref="A54" location="'Application Attribute Testing'!A94" display="DMA02"/>
     <hyperlink ref="A55" location="'Application Attribute Testing'!A95" display="DMA03"/>
     <hyperlink ref="A56" location="'Application Attribute Testing'!A96" display="DMA04"/>
     <hyperlink ref="A60" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="H60" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink ref="I60" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink ref="J60" location="'Application Attribute Testing'!A111" display="E02"/>
+    <hyperlink ref="K60" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="L60" location="'Application Attribute Testing'!A113" display="E04"/>
+    <hyperlink ref="M60" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A64" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink ref="H64" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink ref="I64" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink ref="J64" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink ref="K64" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink ref="L64" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink ref="M64" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink ref="N64" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink ref="O64" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="A68" location="'Application Attribute Testing'!A114" display="E05"/>
+    <hyperlink ref="H68" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink ref="I68" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink ref="J68" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink ref="K68" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink ref="L68" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink ref="M68" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink ref="N68" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="O68" location="'Application Attribute Testing'!A114" display="E05"/>
+    <hyperlink ref="P68" location="'Application Attribute Testing'!A116" display="E08"/>
+    <hyperlink ref="Q68" location="'Application Attribute Testing'!A117" display="E09"/>
+    <hyperlink ref="R68" location="'Application Attribute Testing'!A118" display="E10"/>
     <hyperlink ref="A72" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink ref="H72" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink ref="I72" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink ref="J72" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink ref="K72" location="'Application Attribute Testing'!A111" display="E02"/>
+    <hyperlink ref="L72" location="'Application Attribute Testing'!A114" display="E05"/>
+    <hyperlink ref="M72" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A76" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink ref="H76" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink ref="I76" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink ref="J76" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink ref="K76" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink ref="L76" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink ref="M76" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink ref="N76" location="'Application Attribute Testing'!A93" display="DMA01"/>
+    <hyperlink ref="O76" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink ref="P76" location="'Application Attribute Testing'!A95" display="DMA03"/>
+    <hyperlink ref="Q76" location="'Application Attribute Testing'!A96" display="DMA04"/>
+    <hyperlink ref="R76" location="'Application Attribute Testing'!A97" display="DMA05"/>
+    <hyperlink ref="S76" location="'Application Attribute Testing'!A98" display="DMA06"/>
+    <hyperlink ref="T76" location="'Application Attribute Testing'!A99" display="DMA07"/>
+    <hyperlink ref="U76" location="'Application Attribute Testing'!A100" display="DMA08"/>
+    <hyperlink ref="V76" location="'Application Attribute Testing'!A101" display="DMA09"/>
+    <hyperlink ref="W76" location="'Application Attribute Testing'!A102" display="DMA10"/>
+    <hyperlink ref="X76" location="'Application Attribute Testing'!A103" display="DMA11"/>
+    <hyperlink ref="Y76" location="'Application Attribute Testing'!A104" display="DMA12"/>
+    <hyperlink ref="Z76" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink ref="AA76" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A77" location="'Application Attribute Testing'!A93" display="DMA01"/>
     <hyperlink ref="A78" location="'Application Attribute Testing'!A94" display="DMA02"/>
     <hyperlink ref="A79" location="'Application Attribute Testing'!A95" display="DMA03"/>

</xml_diff>

<commit_message>
Conclusion table: cross-reference evidence refs and attributes per application
For each in-scope application, 'Evidence references' now shows every
ref with the attribute columns it supports (e.g. MA01 -> D, K, N) and
'Attributes tested' shows every attribute with its PASS result and the
refs behind it (e.g. D Application Name - PASS -> MA01, E01, ...),
taken from the original attribute testing. Row heights sized to show
the full lists.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VJjJPWjXw5ntc2ii5NsFQ1
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION.xlsx
+++ b/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION.xlsx
@@ -2059,7 +2059,6 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1" s="73">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -2414,7 +2413,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
@@ -2436,7 +2434,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="77" t="inlineStr">
         <is>
@@ -4902,7 +4899,6 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="33.15" customHeight="1" s="73">
       <c r="A16" s="50" t="inlineStr">
         <is>
@@ -5265,59 +5261,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
     <row r="79" ht="75" customHeight="1" s="73">
       <c r="A79" s="85" t="inlineStr">
         <is>
@@ -11000,7 +10943,7 @@
         </is>
       </c>
     </row>
-    <row r="157" ht="26" customHeight="1" s="73">
+    <row r="157" ht="40" customHeight="1" s="73">
       <c r="A157" s="62" t="inlineStr">
         <is>
           <t>App ID</t>
@@ -11018,12 +10961,12 @@
       </c>
       <c r="D157" s="62" t="inlineStr">
         <is>
-          <t>Evidence references (click App ID for full detail)</t>
+          <t>Evidence references → attributes they support (column letters; click App ID for full detail)</t>
         </is>
       </c>
       <c r="E157" s="62" t="inlineStr">
         <is>
-          <t>Attributes tested</t>
+          <t>Attributes tested → evidence references (PASS)</t>
         </is>
       </c>
       <c r="F157" s="62" t="inlineStr">
@@ -11037,7 +10980,7 @@
         </is>
       </c>
     </row>
-    <row r="158" ht="124" customHeight="1" s="73">
+    <row r="158" ht="258" customHeight="1" s="73">
       <c r="A158" s="70" t="inlineStr">
         <is>
           <t>1822</t>
@@ -11055,12 +10998,36 @@
       </c>
       <c r="D158" s="65" t="inlineStr">
         <is>
-          <t>BLA01, DMA01, DMA02, MA01, E01, E02, E03, E04, E05, E09, E16b</t>
+          <t>BLA01 → B, E, F, I, L, M, O
+DMA01 → G, H, J, O
+DMA02 → B, C, L, M, N
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, K
+E05 → M, N
+E09 → E, G, H, J, M, N, O
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E158" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA01, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA01, E03, E09, E16b
+F Business Data validation – PASS → BLA01, E03, E16b
+G Business line manager name – PASS → DMA01, E03, E09
+H Business line manager approval dates – PASS → DMA01, E03, E09
+I DIV Test procedures listed within the Test results document – PASS → BLA01, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → DMA01, E09
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA01, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA01, DMA02, E03, E05, E09
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05, E09
+O Business Line Approval of Results – PASS → BLA01, DMA01, E03, E09</t>
         </is>
       </c>
       <c r="F158" s="65" t="inlineStr">
@@ -11074,7 +11041,7 @@
         </is>
       </c>
     </row>
-    <row r="159" ht="124" customHeight="1" s="73">
+    <row r="159" ht="258" customHeight="1" s="73">
       <c r="A159" s="70" t="inlineStr">
         <is>
           <t>1867</t>
@@ -11092,12 +11059,36 @@
       </c>
       <c r="D159" s="65" t="inlineStr">
         <is>
-          <t>BLA01, DMA01, DMA02, MA01, E01, E02, E03, E04, E05, E09, E16b</t>
+          <t>BLA01 → B, E, F, I, L, M, O
+DMA01 → G, H, J, O
+DMA02 → B, C, L, M, N
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, E, F, G, H, K
+E05 → M, N
+E09 → E, G, H, J, M, N, O
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E159" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA01, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA01, E03, E04, E09, E16b
+F Business Data validation – PASS → BLA01, E03, E04, E16b
+G Business line manager name – PASS → DMA01, E03, E04, E09
+H Business line manager approval dates – PASS → DMA01, E03, E04, E09
+I DIV Test procedures listed within the Test results document – PASS → BLA01, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → DMA01, E09
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA01, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA01, DMA02, E03, E05, E09
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05, E09
+O Business Line Approval of Results – PASS → BLA01, DMA01, E03, E09</t>
         </is>
       </c>
       <c r="F159" s="65" t="inlineStr">
@@ -11111,7 +11102,7 @@
         </is>
       </c>
     </row>
-    <row r="160" ht="124" customHeight="1" s="73">
+    <row r="160" ht="258" customHeight="1" s="73">
       <c r="A160" s="70" t="inlineStr">
         <is>
           <t>1868</t>
@@ -11129,12 +11120,36 @@
       </c>
       <c r="D160" s="65" t="inlineStr">
         <is>
-          <t>BLA01, DMA01, DMA02, MA01, E01, E02, E03, E04, E05, E09, E16b</t>
+          <t>BLA01 → B, E, F, I, L, M, O
+DMA01 → G, H, J, O
+DMA02 → B, C, L, M, N
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, E, F, G, H, K
+E05 → M, N
+E09 → E, G, H, J, M, N, O
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E160" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA01, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA01, E03, E04, E09, E16b
+F Business Data validation – PASS → BLA01, E03, E04, E16b
+G Business line manager name – PASS → DMA01, E03, E04, E09
+H Business line manager approval dates – PASS → DMA01, E03, E04, E09
+I DIV Test procedures listed within the Test results document – PASS → BLA01, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → DMA01, E09
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA01, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA01, DMA02, E03, E05, E09
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05, E09
+O Business Line Approval of Results – PASS → BLA01, DMA01, E03, E09</t>
         </is>
       </c>
       <c r="F160" s="65" t="inlineStr">
@@ -11148,7 +11163,7 @@
         </is>
       </c>
     </row>
-    <row r="161" ht="124" customHeight="1" s="73">
+    <row r="161" ht="294" customHeight="1" s="73">
       <c r="A161" s="70" t="inlineStr">
         <is>
           <t>3299</t>
@@ -11166,12 +11181,39 @@
       </c>
       <c r="D161" s="65" t="inlineStr">
         <is>
-          <t>BLA01, BLA02, DMA01, DMA02, DMA05, DMA11, MA01, E01, E02, E03, E04, E05, E09, E16b</t>
+          <t>BLA01 → B, E, F, I, L, M, O
+BLA02 → B, E, F, I, L, M, O
+DMA01 → G, H, J, O
+DMA02 → B, C, G, H, J, L, M, N, O
+DMA05 → G, H, J, O
+DMA11 → G, H, J, O
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, E, F, G, H, K
+E05 → M, N
+E09 → E, G, H, J, M, N, O
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E161" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA01, BLA02, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA01, BLA02, E03, E04, E09, E16b
+F Business Data validation – PASS → BLA01, BLA02, E03, E04, E16b
+G Business line manager name – PASS → DMA01, DMA02, DMA05, DMA11, E03, E04, E09
+H Business line manager approval dates – PASS → DMA01, DMA02, DMA05, DMA11, E03, E04, E09
+I DIV Test procedures listed within the Test results document – PASS → BLA01, BLA02, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → DMA01, DMA02, DMA05, DMA11, E09
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA01, BLA02, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA01, BLA02, DMA02, E03, E05, E09
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05, E09
+O Business Line Approval of Results – PASS → BLA01, BLA02, DMA01, DMA02, DMA05, DMA11, E03, E09</t>
         </is>
       </c>
       <c r="F161" s="65" t="inlineStr">
@@ -11185,7 +11227,7 @@
         </is>
       </c>
     </row>
-    <row r="162" ht="124" customHeight="1" s="73">
+    <row r="162" ht="246" customHeight="1" s="73">
       <c r="A162" s="70" t="inlineStr">
         <is>
           <t>4052</t>
@@ -11203,12 +11245,35 @@
       </c>
       <c r="D162" s="65" t="inlineStr">
         <is>
-          <t>BLA04, DMA02, DMA04, MA01, E01, E02, E03, E04, E05, E16b</t>
+          <t>BLA04 → B, E, F, I, L, M, O
+DMA02 → B, C, L, M, N
+DMA04 → G, H, J, O
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, K
+E05 → M, N
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E162" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA04, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA04, E03, E16b
+F Business Data validation – PASS → BLA04, E03, E16b
+G Business line manager name – PASS → DMA04, E03
+H Business line manager approval dates – PASS → DMA04, E03
+I DIV Test procedures listed within the Test results document – PASS → BLA04, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → DMA04
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA04, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA04, DMA02, E03, E05
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05
+O Business Line Approval of Results – PASS → BLA04, DMA04, E03</t>
         </is>
       </c>
       <c r="F162" s="65" t="inlineStr">
@@ -11222,7 +11287,7 @@
         </is>
       </c>
     </row>
-    <row r="163" ht="124" customHeight="1" s="73">
+    <row r="163" ht="246" customHeight="1" s="73">
       <c r="A163" s="70" t="inlineStr">
         <is>
           <t>3301</t>
@@ -11240,12 +11305,37 @@
       </c>
       <c r="D163" s="65" t="inlineStr">
         <is>
-          <t>BLA03, DMA02, DMA03, MA01, E01, E02, E03, E04, E05, E07, E08, E16b</t>
+          <t>BLA03 → B, E, F, I, L, M, O
+DMA02 → B, C, L, M, N
+DMA03 → G, H, J, O
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, K
+E05 → M, N
+E07 → F
+E08 → F, M
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E163" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA03, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA03, E03, E16b
+F Business Data validation – PASS → BLA03, E03, E07, E08, E16b
+G Business line manager name – PASS → DMA03, E03
+H Business line manager approval dates – PASS → DMA03, E03
+I DIV Test procedures listed within the Test results document – PASS → BLA03, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → DMA03
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA03, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA03, DMA02, E03, E05, E08
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05
+O Business Line Approval of Results – PASS → BLA03, DMA03, E03</t>
         </is>
       </c>
       <c r="F163" s="65" t="inlineStr">
@@ -11259,7 +11349,7 @@
         </is>
       </c>
     </row>
-    <row r="164" ht="124" customHeight="1" s="73">
+    <row r="164" ht="282" customHeight="1" s="73">
       <c r="A164" s="70" t="inlineStr">
         <is>
           <t>1903</t>
@@ -11277,12 +11367,39 @@
       </c>
       <c r="D164" s="65" t="inlineStr">
         <is>
-          <t>BLA02, BLA03, DMA02, DMA03, DMA05, MA01, E01, E02, E03, E04, E05, E07, E08, E16b</t>
+          <t>BLA02 → B, E, F, I, L, M, O
+BLA03 → B, E, F, I, L, M, O
+DMA02 → B, C, G, H, J, L, M, N, O
+DMA03 → G, H, J, O
+DMA05 → G, H, J, O
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, E, F, G, H, K
+E05 → M, N
+E07 → F
+E08 → F, M
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E164" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA02, BLA03, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA02, BLA03, E03, E04, E16b
+F Business Data validation – PASS → BLA02, BLA03, E03, E04, E07, E08, E16b
+G Business line manager name – PASS → DMA02, DMA03, DMA05, E03, E04
+H Business line manager approval dates – PASS → DMA02, DMA03, DMA05, E03, E04
+I DIV Test procedures listed within the Test results document – PASS → BLA02, BLA03, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → DMA02, DMA03, DMA05
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA02, BLA03, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA02, BLA03, DMA02, E03, E05, E08
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05
+O Business Line Approval of Results – PASS → BLA02, BLA03, DMA02, DMA03, DMA05, E03</t>
         </is>
       </c>
       <c r="F164" s="65" t="inlineStr">
@@ -11296,7 +11413,7 @@
         </is>
       </c>
     </row>
-    <row r="165" ht="124" customHeight="1" s="73">
+    <row r="165" ht="246" customHeight="1" s="73">
       <c r="A165" s="70" t="inlineStr">
         <is>
           <t>1917</t>
@@ -11314,12 +11431,36 @@
       </c>
       <c r="D165" s="65" t="inlineStr">
         <is>
-          <t>BLA05, BLA06, DMA02, MA01, E01, E02, E03, E04, E05, E10, E16b</t>
+          <t>BLA05 → B, E, F, I, L, M, O
+BLA06 → G, H, J, O
+DMA02 → B, C, L, M, N
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, K
+E05 → M, N
+E10 → M
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E165" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA05, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA05, E03, E16b
+F Business Data validation – PASS → BLA05, E03, E16b
+G Business line manager name – PASS → BLA06, E03
+H Business line manager approval dates – PASS → BLA06, E03
+I DIV Test procedures listed within the Test results document – PASS → BLA05, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → BLA06
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA05, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA05, DMA02, E03, E05, E10
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05
+O Business Line Approval of Results – PASS → BLA05, BLA06, E03</t>
         </is>
       </c>
       <c r="F165" s="65" t="inlineStr">
@@ -11333,7 +11474,7 @@
         </is>
       </c>
     </row>
-    <row r="166" ht="124" customHeight="1" s="73">
+    <row r="166" ht="270" customHeight="1" s="73">
       <c r="A166" s="70" t="inlineStr">
         <is>
           <t>1936</t>
@@ -11351,12 +11492,38 @@
       </c>
       <c r="D166" s="65" t="inlineStr">
         <is>
-          <t>BLA03, BLA04, DMA02, DMA04, MA01, E01, E02, E03, E04, E05, E07, E08, E16b</t>
+          <t>BLA03 → B, E, F, I, L, M, O
+BLA04 → B, E, F, I, L, M, O
+DMA02 → B, C, G, H, J, L, M, N, O
+DMA04 → G, H, J, O
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, E, F, G, H, K
+E05 → M, N
+E07 → F
+E08 → F, M
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E166" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA03, BLA04, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA03, BLA04, E03, E04, E16b
+F Business Data validation – PASS → BLA03, BLA04, E03, E04, E07, E08, E16b
+G Business line manager name – PASS → DMA02, DMA04, E03, E04
+H Business line manager approval dates – PASS → DMA02, DMA04, E03, E04
+I DIV Test procedures listed within the Test results document – PASS → BLA03, BLA04, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → DMA02, DMA04
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA03, BLA04, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA03, BLA04, DMA02, E03, E05, E08
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05
+O Business Line Approval of Results – PASS → BLA03, BLA04, DMA02, DMA04, E03</t>
         </is>
       </c>
       <c r="F166" s="65" t="inlineStr">
@@ -11370,7 +11537,7 @@
         </is>
       </c>
     </row>
-    <row r="167" ht="124" customHeight="1" s="73">
+    <row r="167" ht="378" customHeight="1" s="73">
       <c r="A167" s="70" t="inlineStr">
         <is>
           <t>1937</t>
@@ -11388,12 +11555,54 @@
       </c>
       <c r="D167" s="65" t="inlineStr">
         <is>
-          <t>BLA01, BLA02, BLA03, BLA04, BLA05, BLA06, DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12, MA01, E01, E02, E03, E04, E05, E07, E08, E09, E10, E16b</t>
+          <t>BLA01 → B, E, F, I, L, M, O
+BLA02 → B, E, F, I, L, M, O
+BLA03 → B, E, F, I, L, M, O
+BLA04 → B, E, F, I, L, M, O
+BLA05 → B, E, F, I, L, M, O
+BLA06 → G, H, J, O
+DMA01 → G, H, J, O
+DMA02 → B, C, G, H, J, L, M, N, O
+DMA03 → G, H, J, O
+DMA04 → G, H, J, O
+DMA05 → G, H, J, O
+DMA06 → G, H, J, O
+DMA07 → G, H, J, O
+DMA08 → G, H, J, O
+DMA09 → G, H, J, O
+DMA10 → G, H, J, O
+DMA11 → G, H, J, O
+DMA12 → G, H, J, O
+MA01 → D, K, N
+E01 → D, B, C, K, L, N
+E02 → D, K, N
+E03 → D, B, C, E, F, G, H, I, K, L, M, O
+E04 → D, E, F, G, H, K
+E05 → M, N
+E07 → F
+E08 → F, M
+E09 → G, H, J, O
+E10 → M
+E16b → D, B, E, F, I, K</t>
         </is>
       </c>
       <c r="E167" s="65" t="inlineStr">
         <is>
-          <t>14/14 PASS – D Application Name; B IT DR exercise name; C IT DR exercise name, was the excercise annually executed?; E Business Tester; F Business Data validation; G Business line manager name; H Business line manager approval dates; I DIV Test procedures listed within the Test results document; J Emails showing Business line manager approval of DIV testing results; K All evidence of Data Integrity DR test in BCIC; L Annual Testing Executed; M Data Integrity Validation Performed by IT DR Team; N Applications in Scope Identified; O Business Line Approval of Results</t>
+          <t>14/14 PASS
+D Application Name – PASS → MA01, E01, E02, E03, E04, E16b
+B IT DR exercise name – PASS → BLA01, BLA02, BLA03, BLA04, BLA05, DMA02, E01, E03, E16b
+C IT DR exercise name, was the excercise annually executed? – PASS → DMA02, E01, E03
+E Business Tester – PASS → BLA01, BLA02, BLA03, BLA04, BLA05, E03, E04, E16b
+F Business Data validation – PASS → BLA01, BLA02, BLA03, BLA04, BLA05, E03, E04, E07, E08, E16b
+G Business line manager name – PASS → BLA06, DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12, E03, E04, E09
+H Business line manager approval dates – PASS → BLA06, DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12, E03, E04, E09
+I DIV Test procedures listed within the Test results document – PASS → BLA01, BLA02, BLA03, BLA04, BLA05, E03, E16b
+J Emails showing Business line manager approval of DIV testing results – PASS → BLA06, DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12, E09
+K All evidence of Data Integrity DR test in BCIC – PASS → MA01, E01, E02, E03, E04, E16b
+L Annual Testing Executed – PASS → BLA01, BLA02, BLA03, BLA04, BLA05, DMA02, E01, E03
+M Data Integrity Validation Performed by IT DR Team – PASS → BLA01, BLA02, BLA03, BLA04, BLA05, DMA02, E03, E05, E08, E10
+N Applications in Scope Identified – PASS → DMA02, MA01, E01, E02, E05
+O Business Line Approval of Results – PASS → BLA01, BLA02, BLA03, BLA04, BLA05, BLA06, DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12, E03, E09</t>
         </is>
       </c>
       <c r="F167" s="65" t="inlineStr">
@@ -11818,7 +12027,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="60" customHeight="1" s="73">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -13483,7 +13691,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15.5" customHeight="1" s="73">
       <c r="A16" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Link evidence file paths to the evidence files
Every single evidence file path in 'Application Attribute Testing'
(attribute sections, evidence review, reference table) and every file
name / folder in the Evidence Index is now a relative hyperlink into
BSI.IT.6.C7.3-Evidences, so clicking opens the file (or folder)
directly. Links resolve when the workbook is kept next to the
BSI.IT.6.C7.3-Evidences folder; a note on the column headers says so.
Internal navigation links unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VJjJPWjXw5ntc2ii5NsFQ1
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION.xlsx
+++ b/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION.xlsx
@@ -26,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="39">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -239,6 +239,12 @@
     <font>
       <name val="Carlito"/>
       <b val="1"/>
+      <color rgb="FF0563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Carlito"/>
       <color rgb="FF0563C1"/>
       <sz val="10"/>
       <u val="single"/>
@@ -534,7 +540,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -752,6 +758,9 @@
     </xf>
     <xf numFmtId="0" fontId="36" fillId="10" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1256,6 +1265,36 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>BSI.IT.6.C7.3</author>
+  </authors>
+  <commentList>
+    <comment ref="B22" authorId="0" shapeId="0">
+      <text>
+        <t>Click an evidence file path to open the file. Keep this workbook in the same folder as the 'BSI.IT.6.C7.3-Evidences' folder (e.g. both in the same SharePoint / network / local folder) so the links resolve.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>BSI.IT.6.C7.3</author>
+  </authors>
+  <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>Click an evidence file path to open the file. Keep this workbook in the same folder as the 'BSI.IT.6.C7.3-Evidences' folder (e.g. both in the same SharePoint / network / local folder) so the links resolve.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScopePopulationTable" displayName="ScopePopulationTable" ref="A4:H14" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="8">
@@ -6102,7 +6141,7 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B23" s="65" t="inlineStr">
+      <c r="B23" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
         </is>
@@ -6239,7 +6278,7 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B27" s="65" t="inlineStr">
+      <c r="B27" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
@@ -6384,7 +6423,7 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B32" s="65" t="inlineStr">
+      <c r="B32" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
@@ -6527,7 +6566,7 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B36" s="65" t="inlineStr">
+      <c r="B36" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
@@ -6675,7 +6714,7 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B40" s="65" t="inlineStr">
+      <c r="B40" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
@@ -6853,7 +6892,7 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B44" s="65" t="inlineStr">
+      <c r="B44" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
@@ -7031,7 +7070,7 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B48" s="65" t="inlineStr">
+      <c r="B48" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
@@ -7164,7 +7203,7 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B52" s="65" t="inlineStr">
+      <c r="B52" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
         </is>
@@ -7274,7 +7313,7 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B53" s="65" t="inlineStr">
+      <c r="B53" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
         </is>
@@ -7317,7 +7356,7 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B54" s="65" t="inlineStr">
+      <c r="B54" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
         </is>
@@ -7359,7 +7398,7 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B55" s="65" t="inlineStr">
+      <c r="B55" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
         </is>
@@ -7400,7 +7439,7 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B56" s="65" t="inlineStr">
+      <c r="B56" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
         </is>
@@ -7491,7 +7530,7 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B60" s="65" t="inlineStr">
+      <c r="B60" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
@@ -7619,7 +7658,7 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B64" s="65" t="inlineStr">
+      <c r="B64" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
@@ -7758,7 +7797,7 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B68" s="65" t="inlineStr">
+      <c r="B68" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
         </is>
@@ -7911,7 +7950,7 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B72" s="65" t="inlineStr">
+      <c r="B72" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
         </is>
@@ -8048,7 +8087,7 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B76" s="65" t="inlineStr">
+      <c r="B76" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
         </is>
@@ -8188,7 +8227,7 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B77" s="65" t="inlineStr">
+      <c r="B77" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
         </is>
@@ -8231,7 +8270,7 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B78" s="65" t="inlineStr">
+      <c r="B78" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
         </is>
@@ -8273,7 +8312,7 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B79" s="65" t="inlineStr">
+      <c r="B79" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
         </is>
@@ -8314,7 +8353,7 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B80" s="65" t="inlineStr">
+      <c r="B80" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
         </is>
@@ -8400,7 +8439,7 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B84" s="65" t="inlineStr">
+      <c r="B84" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
         </is>
@@ -8437,7 +8476,7 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B85" s="65" t="inlineStr">
+      <c r="B85" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
         </is>
@@ -8474,7 +8513,7 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B86" s="65" t="inlineStr">
+      <c r="B86" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
         </is>
@@ -8511,7 +8550,7 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B87" s="65" t="inlineStr">
+      <c r="B87" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
         </is>
@@ -8548,7 +8587,7 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B88" s="65" t="inlineStr">
+      <c r="B88" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
         </is>
@@ -8585,7 +8624,7 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B89" s="65" t="inlineStr">
+      <c r="B89" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
         </is>
@@ -8667,7 +8706,7 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B93" s="65" t="inlineStr">
+      <c r="B93" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
         </is>
@@ -8704,7 +8743,7 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B94" s="65" t="inlineStr">
+      <c r="B94" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
         </is>
@@ -8741,7 +8780,7 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B95" s="65" t="inlineStr">
+      <c r="B95" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
         </is>
@@ -8778,7 +8817,7 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B96" s="65" t="inlineStr">
+      <c r="B96" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
         </is>
@@ -8815,7 +8854,7 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B97" s="65" t="inlineStr">
+      <c r="B97" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
         </is>
@@ -8852,7 +8891,7 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B98" s="65" t="inlineStr">
+      <c r="B98" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
         </is>
@@ -8889,7 +8928,7 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B99" s="65" t="inlineStr">
+      <c r="B99" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
         </is>
@@ -8926,7 +8965,7 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B100" s="65" t="inlineStr">
+      <c r="B100" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
         </is>
@@ -8963,7 +9002,7 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B101" s="65" t="inlineStr">
+      <c r="B101" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
         </is>
@@ -9000,7 +9039,7 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B102" s="65" t="inlineStr">
+      <c r="B102" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
         </is>
@@ -9037,7 +9076,7 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B103" s="65" t="inlineStr">
+      <c r="B103" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
         </is>
@@ -9074,7 +9113,7 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B104" s="65" t="inlineStr">
+      <c r="B104" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
         </is>
@@ -9111,7 +9150,7 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B105" s="65" t="inlineStr">
+      <c r="B105" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
         </is>
@@ -9193,7 +9232,7 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B109" s="65" t="inlineStr">
+      <c r="B109" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
         </is>
@@ -9230,7 +9269,7 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B110" s="65" t="inlineStr">
+      <c r="B110" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
@@ -9267,7 +9306,7 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B111" s="65" t="inlineStr">
+      <c r="B111" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
         </is>
@@ -9304,7 +9343,7 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B112" s="65" t="inlineStr">
+      <c r="B112" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
@@ -9341,7 +9380,7 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B113" s="65" t="inlineStr">
+      <c r="B113" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
         </is>
@@ -9378,7 +9417,7 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B114" s="65" t="inlineStr">
+      <c r="B114" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
         </is>
@@ -9415,7 +9454,7 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B115" s="65" t="inlineStr">
+      <c r="B115" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
         </is>
@@ -9452,7 +9491,7 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B116" s="65" t="inlineStr">
+      <c r="B116" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
         </is>
@@ -9489,7 +9528,7 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B117" s="65" t="inlineStr">
+      <c r="B117" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
         </is>
@@ -9526,7 +9565,7 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B118" s="65" t="inlineStr">
+      <c r="B118" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
         </is>
@@ -9563,7 +9602,7 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B119" s="65" t="inlineStr">
+      <c r="B119" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
         </is>
@@ -9600,7 +9639,7 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B120" s="65" t="inlineStr">
+      <c r="B120" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
         </is>
@@ -9682,7 +9721,7 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B124" s="65" t="inlineStr">
+      <c r="B124" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
         </is>
@@ -9725,7 +9764,7 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B125" s="65" t="inlineStr">
+      <c r="B125" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
         </is>
@@ -9768,7 +9807,7 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B126" s="65" t="inlineStr">
+      <c r="B126" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
         </is>
@@ -9811,7 +9850,7 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B127" s="65" t="inlineStr">
+      <c r="B127" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
         </is>
@@ -9854,7 +9893,7 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B128" s="65" t="inlineStr">
+      <c r="B128" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
         </is>
@@ -9897,7 +9936,7 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B129" s="65" t="inlineStr">
+      <c r="B129" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
         </is>
@@ -9937,7 +9976,7 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B130" s="65" t="inlineStr">
+      <c r="B130" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
         </is>
@@ -9977,7 +10016,7 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B131" s="65" t="inlineStr">
+      <c r="B131" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
         </is>
@@ -10022,7 +10061,7 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B132" s="65" t="inlineStr">
+      <c r="B132" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
         </is>
@@ -10062,7 +10101,7 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B133" s="65" t="inlineStr">
+      <c r="B133" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
         </is>
@@ -10102,7 +10141,7 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B134" s="65" t="inlineStr">
+      <c r="B134" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
         </is>
@@ -10142,7 +10181,7 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B135" s="65" t="inlineStr">
+      <c r="B135" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
         </is>
@@ -10182,7 +10221,7 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B136" s="65" t="inlineStr">
+      <c r="B136" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
         </is>
@@ -10222,7 +10261,7 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B137" s="65" t="inlineStr">
+      <c r="B137" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
         </is>
@@ -10262,7 +10301,7 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B138" s="65" t="inlineStr">
+      <c r="B138" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
         </is>
@@ -10302,7 +10341,7 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B139" s="65" t="inlineStr">
+      <c r="B139" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
         </is>
@@ -10342,7 +10381,7 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B140" s="65" t="inlineStr">
+      <c r="B140" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
         </is>
@@ -10382,7 +10421,7 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B141" s="65" t="inlineStr">
+      <c r="B141" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
         </is>
@@ -10422,7 +10461,7 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B142" s="65" t="inlineStr">
+      <c r="B142" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
         </is>
@@ -10459,7 +10498,7 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B143" s="65" t="inlineStr">
+      <c r="B143" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
         </is>
@@ -10498,7 +10537,7 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B144" s="65" t="inlineStr">
+      <c r="B144" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
@@ -10540,7 +10579,7 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B145" s="65" t="inlineStr">
+      <c r="B145" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
         </is>
@@ -10579,7 +10618,7 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B146" s="65" t="inlineStr">
+      <c r="B146" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
@@ -10627,7 +10666,7 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B147" s="65" t="inlineStr">
+      <c r="B147" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
         </is>
@@ -10669,7 +10708,7 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B148" s="65" t="inlineStr">
+      <c r="B148" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
         </is>
@@ -10707,7 +10746,7 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B149" s="65" t="inlineStr">
+      <c r="B149" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
         </is>
@@ -10744,7 +10783,7 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B150" s="65" t="inlineStr">
+      <c r="B150" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
         </is>
@@ -10782,7 +10821,7 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B151" s="65" t="inlineStr">
+      <c r="B151" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
         </is>
@@ -10825,7 +10864,7 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B152" s="65" t="inlineStr">
+      <c r="B152" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
         </is>
@@ -10862,7 +10901,7 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B153" s="65" t="inlineStr">
+      <c r="B153" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
         </is>
@@ -10899,7 +10938,7 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B154" s="65" t="inlineStr">
+      <c r="B154" s="64" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
         </is>
@@ -11782,6 +11821,7 @@
     <hyperlink ref="B18" location="'Application Attribute Testing'!A122" display="Evidence reference table – evidence number → attribute tests"/>
     <hyperlink ref="B19" location="'Application Attribute Testing'!A156" display="Conclusion – all applications in scope (PASS) with evidence references"/>
     <hyperlink ref="A23" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" tooltip="Open evidence file" r:id="rId1"/>
     <hyperlink ref="H23" location="'Application Attribute Testing'!A109" display="MA01"/>
     <hyperlink ref="I23" location="'Application Attribute Testing'!A110" display="E01"/>
     <hyperlink ref="J23" location="'Application Attribute Testing'!A111" display="E02"/>
@@ -11789,6 +11829,7 @@
     <hyperlink ref="L23" location="'Application Attribute Testing'!A113" display="E04"/>
     <hyperlink ref="M23" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A27" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" tooltip="Open evidence file" r:id="rId2"/>
     <hyperlink ref="H27" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I27" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J27" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11799,6 +11840,7 @@
     <hyperlink ref="O27" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="P27" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A32" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" tooltip="Open evidence file" r:id="rId3"/>
     <hyperlink ref="H32" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I32" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J32" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11809,6 +11851,7 @@
     <hyperlink ref="O32" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="P32" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A36" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" tooltip="Open evidence file" r:id="rId4"/>
     <hyperlink ref="H36" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I36" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J36" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11820,6 +11863,7 @@
     <hyperlink ref="P36" location="'Application Attribute Testing'!A116" display="E08"/>
     <hyperlink ref="Q36" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A40" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" tooltip="Open evidence file" r:id="rId5"/>
     <hyperlink ref="H40" location="'Application Attribute Testing'!A89" display="BLA06"/>
     <hyperlink ref="I40" location="'Application Attribute Testing'!A93" display="DMA01"/>
     <hyperlink ref="J40" location="'Application Attribute Testing'!A94" display="DMA02"/>
@@ -11837,6 +11881,7 @@
     <hyperlink ref="V40" location="'Application Attribute Testing'!A113" display="E04"/>
     <hyperlink ref="W40" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A44" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" tooltip="Open evidence file" r:id="rId6"/>
     <hyperlink ref="H44" location="'Application Attribute Testing'!A89" display="BLA06"/>
     <hyperlink ref="I44" location="'Application Attribute Testing'!A93" display="DMA01"/>
     <hyperlink ref="J44" location="'Application Attribute Testing'!A94" display="DMA02"/>
@@ -11854,6 +11899,7 @@
     <hyperlink ref="V44" location="'Application Attribute Testing'!A113" display="E04"/>
     <hyperlink ref="W44" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A48" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" tooltip="Open evidence file" r:id="rId7"/>
     <hyperlink ref="H48" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I48" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J48" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11862,6 +11908,7 @@
     <hyperlink ref="M48" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="N48" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A52" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" tooltip="Open evidence file" r:id="rId8"/>
     <hyperlink ref="H52" location="'Application Attribute Testing'!A89" display="BLA06"/>
     <hyperlink ref="I52" location="'Application Attribute Testing'!A93" display="DMA01"/>
     <hyperlink ref="J52" location="'Application Attribute Testing'!A94" display="DMA02"/>
@@ -11877,10 +11924,15 @@
     <hyperlink ref="T52" location="'Application Attribute Testing'!A104" display="DMA12"/>
     <hyperlink ref="U52" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A53" location="'Application Attribute Testing'!A93" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" tooltip="Open evidence file" r:id="rId9"/>
     <hyperlink ref="A54" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" tooltip="Open evidence file" r:id="rId10"/>
     <hyperlink ref="A55" location="'Application Attribute Testing'!A95" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" tooltip="Open evidence file" r:id="rId11"/>
     <hyperlink ref="A56" location="'Application Attribute Testing'!A96" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" tooltip="Open evidence file" r:id="rId12"/>
     <hyperlink ref="A60" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" tooltip="Open evidence file" r:id="rId13"/>
     <hyperlink ref="H60" location="'Application Attribute Testing'!A109" display="MA01"/>
     <hyperlink ref="I60" location="'Application Attribute Testing'!A110" display="E01"/>
     <hyperlink ref="J60" location="'Application Attribute Testing'!A111" display="E02"/>
@@ -11888,6 +11940,7 @@
     <hyperlink ref="L60" location="'Application Attribute Testing'!A113" display="E04"/>
     <hyperlink ref="M60" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A64" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" tooltip="Open evidence file" r:id="rId14"/>
     <hyperlink ref="H64" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I64" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J64" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11897,6 +11950,7 @@
     <hyperlink ref="N64" location="'Application Attribute Testing'!A110" display="E01"/>
     <hyperlink ref="O64" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="A68" location="'Application Attribute Testing'!A114" display="E05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" tooltip="Open evidence file" r:id="rId15"/>
     <hyperlink ref="H68" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I68" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J68" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11909,6 +11963,7 @@
     <hyperlink ref="Q68" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="R68" location="'Application Attribute Testing'!A118" display="E10"/>
     <hyperlink ref="A72" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" tooltip="Open evidence file" r:id="rId16"/>
     <hyperlink ref="H72" location="'Application Attribute Testing'!A94" display="DMA02"/>
     <hyperlink ref="I72" location="'Application Attribute Testing'!A109" display="MA01"/>
     <hyperlink ref="J72" location="'Application Attribute Testing'!A110" display="E01"/>
@@ -11916,6 +11971,7 @@
     <hyperlink ref="L72" location="'Application Attribute Testing'!A114" display="E05"/>
     <hyperlink ref="M72" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A76" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" tooltip="Open evidence file" r:id="rId17"/>
     <hyperlink ref="H76" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I76" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J76" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11937,40 +11993,106 @@
     <hyperlink ref="Z76" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="AA76" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A77" location="'Application Attribute Testing'!A93" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" tooltip="Open evidence file" r:id="rId18"/>
     <hyperlink ref="A78" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" tooltip="Open evidence file" r:id="rId19"/>
     <hyperlink ref="A79" location="'Application Attribute Testing'!A95" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" tooltip="Open evidence file" r:id="rId20"/>
     <hyperlink ref="A80" location="'Application Attribute Testing'!A96" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" tooltip="Open evidence file" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" tooltip="Open evidence file" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B85" tooltip="Open evidence file" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" tooltip="Open evidence file" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" tooltip="Open evidence file" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" tooltip="Open evidence file" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" tooltip="Open evidence file" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" tooltip="Open evidence file" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" tooltip="Open evidence file" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" tooltip="Open evidence file" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" tooltip="Open evidence file" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" tooltip="Open evidence file" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" tooltip="Open evidence file" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" tooltip="Open evidence file" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" tooltip="Open evidence file" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" tooltip="Open evidence file" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" tooltip="Open evidence file" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" tooltip="Open evidence file" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" tooltip="Open evidence file" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B105" tooltip="Open evidence file" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" tooltip="Open evidence file" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" tooltip="Open evidence file" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" tooltip="Open evidence file" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" tooltip="Open evidence file" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" tooltip="Open evidence file" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" tooltip="Open evidence file" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" tooltip="Open evidence file" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" tooltip="Open evidence file" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B117" tooltip="Open evidence file" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" tooltip="Open evidence file" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B119" tooltip="Open evidence file" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" tooltip="Open evidence file" r:id="rId52"/>
     <hyperlink ref="A124" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" tooltip="Open evidence file" r:id="rId53"/>
     <hyperlink ref="A125" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" tooltip="Open evidence file" r:id="rId54"/>
     <hyperlink ref="A126" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" tooltip="Open evidence file" r:id="rId55"/>
     <hyperlink ref="A127" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" tooltip="Open evidence file" r:id="rId56"/>
     <hyperlink ref="A128" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" tooltip="Open evidence file" r:id="rId57"/>
     <hyperlink ref="A129" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" tooltip="Open evidence file" r:id="rId58"/>
     <hyperlink ref="A130" location="'Application Attribute Testing'!A93" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" tooltip="Open evidence file" r:id="rId59"/>
     <hyperlink ref="A131" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" tooltip="Open evidence file" r:id="rId60"/>
     <hyperlink ref="A132" location="'Application Attribute Testing'!A95" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B132" tooltip="Open evidence file" r:id="rId61"/>
     <hyperlink ref="A133" location="'Application Attribute Testing'!A96" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B133" tooltip="Open evidence file" r:id="rId62"/>
     <hyperlink ref="A134" location="'Application Attribute Testing'!A97" display="DMA05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B134" tooltip="Open evidence file" r:id="rId63"/>
     <hyperlink ref="A135" location="'Application Attribute Testing'!A98" display="DMA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B135" tooltip="Open evidence file" r:id="rId64"/>
     <hyperlink ref="A136" location="'Application Attribute Testing'!A99" display="DMA07"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B136" tooltip="Open evidence file" r:id="rId65"/>
     <hyperlink ref="A137" location="'Application Attribute Testing'!A100" display="DMA08"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B137" tooltip="Open evidence file" r:id="rId66"/>
     <hyperlink ref="A138" location="'Application Attribute Testing'!A101" display="DMA09"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" tooltip="Open evidence file" r:id="rId67"/>
     <hyperlink ref="A139" location="'Application Attribute Testing'!A102" display="DMA10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" tooltip="Open evidence file" r:id="rId68"/>
     <hyperlink ref="A140" location="'Application Attribute Testing'!A103" display="DMA11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" tooltip="Open evidence file" r:id="rId69"/>
     <hyperlink ref="A141" location="'Application Attribute Testing'!A104" display="DMA12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B141" tooltip="Open evidence file" r:id="rId70"/>
     <hyperlink ref="A142" location="'Application Attribute Testing'!A105" display="DMA13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B142" tooltip="Open evidence file" r:id="rId71"/>
     <hyperlink ref="A143" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" tooltip="Open evidence file" r:id="rId72"/>
     <hyperlink ref="A144" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" tooltip="Open evidence file" r:id="rId73"/>
     <hyperlink ref="A145" location="'Application Attribute Testing'!A111" display="E02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" tooltip="Open evidence file" r:id="rId74"/>
     <hyperlink ref="A146" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B146" tooltip="Open evidence file" r:id="rId75"/>
     <hyperlink ref="A147" location="'Application Attribute Testing'!A113" display="E04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" tooltip="Open evidence file" r:id="rId76"/>
     <hyperlink ref="A148" location="'Application Attribute Testing'!A114" display="E05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" tooltip="Open evidence file" r:id="rId77"/>
     <hyperlink ref="A149" location="'Application Attribute Testing'!A115" display="E07"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" tooltip="Open evidence file" r:id="rId78"/>
     <hyperlink ref="A150" location="'Application Attribute Testing'!A116" display="E08"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B150" tooltip="Open evidence file" r:id="rId79"/>
     <hyperlink ref="A151" location="'Application Attribute Testing'!A117" display="E09"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B151" tooltip="Open evidence file" r:id="rId80"/>
     <hyperlink ref="A152" location="'Application Attribute Testing'!A118" display="E10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B152" tooltip="Open evidence file" r:id="rId81"/>
     <hyperlink ref="A153" location="'Application Attribute Testing'!A119" display="E13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B153" tooltip="Open evidence file" r:id="rId82"/>
     <hyperlink ref="A154" location="'Application Attribute Testing'!A120" display="E16b"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B154" tooltip="Open evidence file" r:id="rId83"/>
     <hyperlink ref="A158" location="'Application Attribute Testing-1'!A3" display="1822"/>
     <hyperlink ref="B158" location="'Application Attribute Testing-1'!A3" display="ACH Express"/>
     <hyperlink ref="A159" location="'Application Attribute Testing-1'!A4" display="1867"/>
@@ -11994,6 +12116,7 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -13876,12 +13999,12 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B3" s="35" t="inlineStr">
+      <c r="B3" s="92" t="inlineStr">
         <is>
           <t>MA01_BSI In-Scope Applications-2026.png</t>
         </is>
       </c>
-      <c r="C3" s="35" t="inlineStr">
+      <c r="C3" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications</t>
         </is>
@@ -13930,12 +14053,12 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B4" s="35" t="inlineStr">
+      <c r="B4" s="92" t="inlineStr">
         <is>
           <t>BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
         </is>
       </c>
-      <c r="C4" s="35" t="inlineStr">
+      <c r="C4" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
         </is>
@@ -13984,12 +14107,12 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B5" s="35" t="inlineStr">
+      <c r="B5" s="92" t="inlineStr">
         <is>
           <t>BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
         </is>
       </c>
-      <c r="C5" s="35" t="inlineStr">
+      <c r="C5" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
         </is>
@@ -14038,12 +14161,12 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B6" s="35" t="inlineStr">
+      <c r="B6" s="92" t="inlineStr">
         <is>
           <t>BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
         </is>
       </c>
-      <c r="C6" s="35" t="inlineStr">
+      <c r="C6" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
         </is>
@@ -14092,12 +14215,12 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B7" s="35" t="inlineStr">
+      <c r="B7" s="92" t="inlineStr">
         <is>
           <t>BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
         </is>
       </c>
-      <c r="C7" s="35" t="inlineStr">
+      <c r="C7" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
         </is>
@@ -14146,12 +14269,12 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B8" s="35" t="inlineStr">
+      <c r="B8" s="92" t="inlineStr">
         <is>
           <t>BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
         </is>
       </c>
-      <c r="C8" s="35" t="inlineStr">
+      <c r="C8" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
         </is>
@@ -14200,12 +14323,12 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B9" s="35" t="inlineStr">
+      <c r="B9" s="92" t="inlineStr">
         <is>
           <t>BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
         </is>
       </c>
-      <c r="C9" s="35" t="inlineStr">
+      <c r="C9" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
         </is>
@@ -14254,12 +14377,12 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B10" s="35" t="inlineStr">
+      <c r="B10" s="92" t="inlineStr">
         <is>
           <t>DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
         </is>
       </c>
-      <c r="C10" s="35" t="inlineStr">
+      <c r="C10" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14308,12 +14431,12 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B11" s="92" t="inlineStr">
         <is>
           <t>DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
         </is>
       </c>
-      <c r="C11" s="35" t="inlineStr">
+      <c r="C11" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14362,12 +14485,12 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B12" s="35" t="inlineStr">
+      <c r="B12" s="92" t="inlineStr">
         <is>
           <t>DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
         </is>
       </c>
-      <c r="C12" s="35" t="inlineStr">
+      <c r="C12" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14416,12 +14539,12 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B13" s="35" t="inlineStr">
+      <c r="B13" s="92" t="inlineStr">
         <is>
           <t>DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
         </is>
       </c>
-      <c r="C13" s="35" t="inlineStr">
+      <c r="C13" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14470,12 +14593,12 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B14" s="35" t="inlineStr">
+      <c r="B14" s="92" t="inlineStr">
         <is>
           <t>DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
         </is>
       </c>
-      <c r="C14" s="35" t="inlineStr">
+      <c r="C14" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14524,12 +14647,12 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B15" s="35" t="inlineStr">
+      <c r="B15" s="92" t="inlineStr">
         <is>
           <t>DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
         </is>
       </c>
-      <c r="C15" s="35" t="inlineStr">
+      <c r="C15" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14578,12 +14701,12 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B16" s="35" t="inlineStr">
+      <c r="B16" s="92" t="inlineStr">
         <is>
           <t>DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
         </is>
       </c>
-      <c r="C16" s="35" t="inlineStr">
+      <c r="C16" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14632,12 +14755,12 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B17" s="35" t="inlineStr">
+      <c r="B17" s="92" t="inlineStr">
         <is>
           <t>DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
         </is>
       </c>
-      <c r="C17" s="35" t="inlineStr">
+      <c r="C17" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14686,12 +14809,12 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B18" s="35" t="inlineStr">
+      <c r="B18" s="92" t="inlineStr">
         <is>
           <t>DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
         </is>
       </c>
-      <c r="C18" s="35" t="inlineStr">
+      <c r="C18" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14740,12 +14863,12 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B19" s="35" t="inlineStr">
+      <c r="B19" s="92" t="inlineStr">
         <is>
           <t>DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
         </is>
       </c>
-      <c r="C19" s="35" t="inlineStr">
+      <c r="C19" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14794,12 +14917,12 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B20" s="35" t="inlineStr">
+      <c r="B20" s="92" t="inlineStr">
         <is>
           <t>DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
         </is>
       </c>
-      <c r="C20" s="35" t="inlineStr">
+      <c r="C20" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14848,12 +14971,12 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B21" s="35" t="inlineStr">
+      <c r="B21" s="92" t="inlineStr">
         <is>
           <t>DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
         </is>
       </c>
-      <c r="C21" s="35" t="inlineStr">
+      <c r="C21" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14902,12 +15025,12 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B22" s="35" t="inlineStr">
+      <c r="B22" s="92" t="inlineStr">
         <is>
           <t>DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
         </is>
       </c>
-      <c r="C22" s="35" t="inlineStr">
+      <c r="C22" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
@@ -14956,12 +15079,12 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B23" s="35" t="inlineStr">
+      <c r="B23" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
       </c>
-      <c r="C23" s="35" t="inlineStr">
+      <c r="C23" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15010,12 +15133,12 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B24" s="35" t="inlineStr">
+      <c r="B24" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
         </is>
       </c>
-      <c r="C24" s="35" t="inlineStr">
+      <c r="C24" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15064,12 +15187,12 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B25" s="35" t="inlineStr">
+      <c r="B25" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
       </c>
-      <c r="C25" s="35" t="inlineStr">
+      <c r="C25" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15118,12 +15241,12 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B26" s="35" t="inlineStr">
+      <c r="B26" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
         </is>
       </c>
-      <c r="C26" s="35" t="inlineStr">
+      <c r="C26" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15172,12 +15295,12 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B27" s="35" t="inlineStr">
+      <c r="B27" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
         </is>
       </c>
-      <c r="C27" s="35" t="inlineStr">
+      <c r="C27" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15226,12 +15349,12 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B28" s="35" t="inlineStr">
+      <c r="B28" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
         </is>
       </c>
-      <c r="C28" s="35" t="inlineStr">
+      <c r="C28" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15280,12 +15403,12 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B29" s="35" t="inlineStr">
+      <c r="B29" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
         </is>
       </c>
-      <c r="C29" s="35" t="inlineStr">
+      <c r="C29" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15334,12 +15457,12 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B30" s="35" t="inlineStr">
+      <c r="B30" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
         </is>
       </c>
-      <c r="C30" s="35" t="inlineStr">
+      <c r="C30" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15388,12 +15511,12 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B31" s="35" t="inlineStr">
+      <c r="B31" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
         </is>
       </c>
-      <c r="C31" s="35" t="inlineStr">
+      <c r="C31" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15442,12 +15565,12 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B32" s="35" t="inlineStr">
+      <c r="B32" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
         </is>
       </c>
-      <c r="C32" s="35" t="inlineStr">
+      <c r="C32" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -15496,12 +15619,12 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B33" s="35" t="inlineStr">
+      <c r="B33" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
         </is>
       </c>
-      <c r="C33" s="35" t="inlineStr">
+      <c r="C33" s="92" t="inlineStr">
         <is>
           <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
         </is>
@@ -17250,38 +17373,101 @@
   <autoFilter ref="A2:K33"/>
   <hyperlinks>
     <hyperlink ref="A3" location="'Application Attribute Testing'!A109" display="MA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" tooltip="Open evidence file" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" tooltip="Open evidence folder" r:id="rId2"/>
     <hyperlink ref="A4" location="'Application Attribute Testing'!A84" display="BLA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" tooltip="Open evidence file" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" tooltip="Open evidence folder" r:id="rId4"/>
     <hyperlink ref="A5" location="'Application Attribute Testing'!A85" display="BLA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" tooltip="Open evidence file" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" tooltip="Open evidence folder" r:id="rId6"/>
     <hyperlink ref="A6" location="'Application Attribute Testing'!A86" display="BLA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" tooltip="Open evidence file" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" tooltip="Open evidence folder" r:id="rId8"/>
     <hyperlink ref="A7" location="'Application Attribute Testing'!A87" display="BLA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" tooltip="Open evidence file" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" tooltip="Open evidence folder" r:id="rId10"/>
     <hyperlink ref="A8" location="'Application Attribute Testing'!A88" display="BLA05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" tooltip="Open evidence file" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" tooltip="Open evidence folder" r:id="rId12"/>
     <hyperlink ref="A9" location="'Application Attribute Testing'!A89" display="BLA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" tooltip="Open evidence file" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" tooltip="Open evidence folder" r:id="rId14"/>
     <hyperlink ref="A10" location="'Application Attribute Testing'!A93" display="DMA01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" tooltip="Open evidence file" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" tooltip="Open evidence folder" r:id="rId16"/>
     <hyperlink ref="A11" location="'Application Attribute Testing'!A94" display="DMA02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" tooltip="Open evidence file" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" tooltip="Open evidence folder" r:id="rId18"/>
     <hyperlink ref="A12" location="'Application Attribute Testing'!A95" display="DMA03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" tooltip="Open evidence file" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" tooltip="Open evidence folder" r:id="rId20"/>
     <hyperlink ref="A13" location="'Application Attribute Testing'!A96" display="DMA04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" tooltip="Open evidence file" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" tooltip="Open evidence folder" r:id="rId22"/>
     <hyperlink ref="A14" location="'Application Attribute Testing'!A97" display="DMA05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" tooltip="Open evidence file" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" tooltip="Open evidence folder" r:id="rId24"/>
     <hyperlink ref="A15" location="'Application Attribute Testing'!A98" display="DMA06"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" tooltip="Open evidence file" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" tooltip="Open evidence folder" r:id="rId26"/>
     <hyperlink ref="A16" location="'Application Attribute Testing'!A99" display="DMA07"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" tooltip="Open evidence file" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" tooltip="Open evidence folder" r:id="rId28"/>
     <hyperlink ref="A17" location="'Application Attribute Testing'!A100" display="DMA08"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" tooltip="Open evidence file" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" tooltip="Open evidence folder" r:id="rId30"/>
     <hyperlink ref="A18" location="'Application Attribute Testing'!A101" display="DMA09"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" tooltip="Open evidence file" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" tooltip="Open evidence folder" r:id="rId32"/>
     <hyperlink ref="A19" location="'Application Attribute Testing'!A102" display="DMA10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" tooltip="Open evidence file" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" tooltip="Open evidence folder" r:id="rId34"/>
     <hyperlink ref="A20" location="'Application Attribute Testing'!A103" display="DMA11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" tooltip="Open evidence file" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" tooltip="Open evidence folder" r:id="rId36"/>
     <hyperlink ref="A21" location="'Application Attribute Testing'!A104" display="DMA12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" tooltip="Open evidence file" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" tooltip="Open evidence folder" r:id="rId38"/>
     <hyperlink ref="A22" location="'Application Attribute Testing'!A105" display="DMA13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" tooltip="Open evidence file" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" tooltip="Open evidence folder" r:id="rId40"/>
     <hyperlink ref="A23" location="'Application Attribute Testing'!A110" display="E01"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" tooltip="Open evidence file" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" tooltip="Open evidence folder" r:id="rId42"/>
     <hyperlink ref="A24" location="'Application Attribute Testing'!A111" display="E02"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" tooltip="Open evidence file" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" tooltip="Open evidence folder" r:id="rId44"/>
     <hyperlink ref="A25" location="'Application Attribute Testing'!A112" display="E03"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" tooltip="Open evidence file" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" tooltip="Open evidence folder" r:id="rId46"/>
     <hyperlink ref="A26" location="'Application Attribute Testing'!A113" display="E04"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" tooltip="Open evidence file" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" tooltip="Open evidence folder" r:id="rId48"/>
     <hyperlink ref="A27" location="'Application Attribute Testing'!A114" display="E05"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" tooltip="Open evidence file" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" tooltip="Open evidence folder" r:id="rId50"/>
     <hyperlink ref="A28" location="'Application Attribute Testing'!A115" display="E07"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" tooltip="Open evidence file" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" tooltip="Open evidence folder" r:id="rId52"/>
     <hyperlink ref="A29" location="'Application Attribute Testing'!A116" display="E08"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" tooltip="Open evidence file" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" tooltip="Open evidence folder" r:id="rId54"/>
     <hyperlink ref="A30" location="'Application Attribute Testing'!A117" display="E09"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" tooltip="Open evidence file" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" tooltip="Open evidence folder" r:id="rId56"/>
     <hyperlink ref="A31" location="'Application Attribute Testing'!A118" display="E10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" tooltip="Open evidence file" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" tooltip="Open evidence folder" r:id="rId58"/>
     <hyperlink ref="A32" location="'Application Attribute Testing'!A119" display="E13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" tooltip="Open evidence file" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" tooltip="Open evidence folder" r:id="rId60"/>
     <hyperlink ref="A33" location="'Application Attribute Testing'!A120" display="E16b"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" tooltip="Open evidence file" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" tooltip="Open evidence folder" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Evidence file links: resolve from a configurable evidence folder
Static relative file links failed ('Cannot open the specified file')
when the workbook was opened away from the evidence folder. All 145
file links are now HYPERLINK() formulas built from the name
EvidenceRoot, set on 'WP Summary' row 27: blank = the
BSI.IT.6.C7.3-Evidences folder next to the saved workbook; otherwise the
pasted local, network or SharePoint path. Row 28 shows the resolved
path and a test link that opens the evidence folder. Workbook set to
recalculate on open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VJjJPWjXw5ntc2ii5NsFQ1
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION.xlsx
+++ b/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION.xlsx
@@ -15,6 +15,8 @@
     <sheet name="DR 2024 Testing Results" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="EvidenceFolder">'WP Summary'!$B$27</definedName>
+    <definedName name="EvidenceRoot">IF(LEN(TRIM(EvidenceFolder))=0,LEFT(CELL("filename",'WP Summary'!$A$1),FIND("[",CELL("filename",'WP Summary'!$A$1))-1)&amp;"BSI.IT.6.C7.3-Evidences"&amp;IF(LEFT(LEFT(CELL("filename",'WP Summary'!$A$1),FIND("[",CELL("filename",'WP Summary'!$A$1))-1),4)="http","/","\"),TRIM(EvidenceFolder)&amp;IF(OR(RIGHT(TRIM(EvidenceFolder),1)="\",RIGHT(TRIM(EvidenceFolder),1)="/"),"",IF(LEFT(TRIM(EvidenceFolder),4)="http","/","\")))</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BSI.IT.6.C7.3 Evidence Index'!$A$2:$K$33</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -26,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="41">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -249,8 +251,18 @@
       <sz val="10"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Carlito"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Carlito"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -361,8 +373,13 @@
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="18">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -536,11 +553,55 @@
         <color rgb="FFBFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -762,6 +823,16 @@
     <xf numFmtId="0" fontId="38" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="21" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1271,9 +1342,9 @@
     <author>BSI.IT.6.C7.3</author>
   </authors>
   <commentList>
-    <comment ref="B22" authorId="0" shapeId="0">
+    <comment ref="B27" authorId="0" shapeId="0">
       <text>
-        <t>Click an evidence file path to open the file. Keep this workbook in the same folder as the 'BSI.IT.6.C7.3-Evidences' folder (e.g. both in the same SharePoint / network / local folder) so the links resolve.</t>
+        <t>Leave blank if the folder 'BSI.IT.6.C7.3-Evidences' is saved next to this workbook. Otherwise paste the full path of the BSI.IT.6.C7.3-Evidences folder, e.g. C:\Audit\BSI.IT.6.C7.3-Evidences  or  \\server\share\BSI.IT.6.C7.3-Evidences  or  https://tenant.sharepoint.com/sites/Audit/Shared Documents/BSI.IT.6.C7.3-Evidences</t>
       </text>
     </comment>
   </commentList>
@@ -1286,9 +1357,24 @@
     <author>BSI.IT.6.C7.3</author>
   </authors>
   <commentList>
+    <comment ref="B22" authorId="0" shapeId="0">
+      <text>
+        <t>Click an evidence file path to open the file. The evidence folder location is set on tab 'WP Summary' (yellow cell, row 27): blank = folder 'BSI.IT.6.C7.3-Evidences' next to this workbook.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>BSI.IT.6.C7.3</author>
+  </authors>
+  <commentList>
     <comment ref="B2" authorId="0" shapeId="0">
       <text>
-        <t>Click an evidence file path to open the file. Keep this workbook in the same folder as the 'BSI.IT.6.C7.3-Evidences' folder (e.g. both in the same SharePoint / network / local folder) so the links resolve.</t>
+        <t>Click an evidence file path to open the file. The evidence folder location is set on tab 'WP Summary' (yellow cell, row 27): blank = folder 'BSI.IT.6.C7.3-Evidences' next to this workbook.</t>
       </text>
     </comment>
   </commentList>
@@ -1529,7 +1615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" style="73" min="1" max="1"/>
@@ -2053,12 +2139,58 @@
     <row r="22" ht="27.15" customHeight="1" s="73"/>
     <row r="23" ht="20.5" customHeight="1" s="73"/>
     <row r="24" ht="20.5" customHeight="1" s="73"/>
+    <row r="26">
+      <c r="A26" s="93" t="inlineStr">
+        <is>
+          <t>Evidence file links – setting (clicking an evidence file path opens the file)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1" s="73">
+      <c r="A27" s="94" t="inlineStr">
+        <is>
+          <t>Evidence folder</t>
+        </is>
+      </c>
+      <c r="B27" s="95" t="n"/>
+      <c r="C27" s="99" t="n"/>
+      <c r="D27" s="99" t="n"/>
+      <c r="E27" s="100" t="n"/>
+      <c r="F27" s="96" t="inlineStr">
+        <is>
+          <t>← Yellow cell: leave blank if the evidence folder sits next to this workbook; otherwise paste its full path (local, network or SharePoint).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="94" t="inlineStr">
+        <is>
+          <t>Links resolve to</t>
+        </is>
+      </c>
+      <c r="B28" s="97">
+        <f>EvidenceRoot</f>
+        <v/>
+      </c>
+      <c r="C28" s="99" t="n"/>
+      <c r="D28" s="99" t="n"/>
+      <c r="E28" s="100" t="n"/>
+      <c r="F28" s="98">
+        <f>HYPERLINK(EvidenceRoot,"▶ Test: open the evidence folder")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="9">
     <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="F28:H28"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A21:H24"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="B28:E28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2069,6 +2201,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -6141,10 +6274,9 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B23" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
-        </is>
+      <c r="B23" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
+        <v/>
       </c>
       <c r="C23" s="65" t="inlineStr">
         <is>
@@ -6278,10 +6410,9 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B27" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
-        </is>
+      <c r="B27" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
+        <v/>
       </c>
       <c r="C27" s="65" t="inlineStr">
         <is>
@@ -6423,10 +6554,9 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B32" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
+      <c r="B32" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
       </c>
       <c r="C32" s="65" t="inlineStr">
         <is>
@@ -6566,10 +6696,9 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B36" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
+      <c r="B36" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
       </c>
       <c r="C36" s="65" t="inlineStr">
         <is>
@@ -6714,10 +6843,9 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B40" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
+      <c r="B40" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
       </c>
       <c r="C40" s="65" t="inlineStr">
         <is>
@@ -6892,10 +7020,9 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B44" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
+      <c r="B44" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
       </c>
       <c r="C44" s="65" t="inlineStr">
         <is>
@@ -7070,10 +7197,9 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B48" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
+      <c r="B48" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
       </c>
       <c r="C48" s="65" t="inlineStr">
         <is>
@@ -7203,10 +7329,9 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B52" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
-        </is>
+      <c r="B52" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
+        <v/>
       </c>
       <c r="C52" s="65" t="inlineStr">
         <is>
@@ -7313,10 +7438,9 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B53" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
-        </is>
+      <c r="B53" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C53" s="65" t="inlineStr">
         <is>
@@ -7356,10 +7480,9 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B54" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
-        </is>
+      <c r="B54" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
+        <v/>
       </c>
       <c r="C54" s="65" t="inlineStr">
         <is>
@@ -7398,10 +7521,9 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B55" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
-        </is>
+      <c r="B55" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C55" s="65" t="inlineStr">
         <is>
@@ -7439,10 +7561,9 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B56" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
-        </is>
+      <c r="B56" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
+        <v/>
       </c>
       <c r="C56" s="65" t="inlineStr">
         <is>
@@ -7530,10 +7651,9 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B60" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
+      <c r="B60" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
       </c>
       <c r="C60" s="65" t="inlineStr">
         <is>
@@ -7658,10 +7778,9 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B64" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
-        </is>
+      <c r="B64" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
+        <v/>
       </c>
       <c r="C64" s="65" t="inlineStr">
         <is>
@@ -7797,10 +7916,9 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B68" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
-        </is>
+      <c r="B68" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
+        <v/>
       </c>
       <c r="C68" s="65" t="inlineStr">
         <is>
@@ -7950,10 +8068,9 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B72" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
-        </is>
+      <c r="B72" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
+        <v/>
       </c>
       <c r="C72" s="65" t="inlineStr">
         <is>
@@ -8087,10 +8204,9 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B76" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
-        </is>
+      <c r="B76" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
+        <v/>
       </c>
       <c r="C76" s="65" t="inlineStr">
         <is>
@@ -8227,10 +8343,9 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B77" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
-        </is>
+      <c r="B77" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C77" s="65" t="inlineStr">
         <is>
@@ -8270,10 +8385,9 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B78" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
-        </is>
+      <c r="B78" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
+        <v/>
       </c>
       <c r="C78" s="65" t="inlineStr">
         <is>
@@ -8312,10 +8426,9 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B79" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
-        </is>
+      <c r="B79" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C79" s="65" t="inlineStr">
         <is>
@@ -8353,10 +8466,9 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B80" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
-        </is>
+      <c r="B80" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
+        <v/>
       </c>
       <c r="C80" s="65" t="inlineStr">
         <is>
@@ -8439,10 +8551,9 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B84" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
-        </is>
+      <c r="B84" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
       </c>
       <c r="C84" s="65" t="inlineStr">
         <is>
@@ -8476,10 +8587,9 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B85" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
-        </is>
+      <c r="B85" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
       </c>
       <c r="C85" s="65" t="inlineStr">
         <is>
@@ -8513,10 +8623,9 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B86" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
-        </is>
+      <c r="B86" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
       </c>
       <c r="C86" s="65" t="inlineStr">
         <is>
@@ -8550,10 +8659,9 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B87" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
-        </is>
+      <c r="B87" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx","\","/"),"02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx")</f>
+        <v/>
       </c>
       <c r="C87" s="65" t="inlineStr">
         <is>
@@ -8587,10 +8695,9 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B88" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
-        </is>
+      <c r="B88" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
       </c>
       <c r="C88" s="65" t="inlineStr">
         <is>
@@ -8624,10 +8731,9 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B89" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
-        </is>
+      <c r="B89" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
+        <v/>
       </c>
       <c r="C89" s="65" t="inlineStr">
         <is>
@@ -8706,10 +8812,9 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B93" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
-        </is>
+      <c r="B93" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C93" s="65" t="inlineStr">
         <is>
@@ -8743,10 +8848,9 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B94" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
-        </is>
+      <c r="B94" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
+        <v/>
       </c>
       <c r="C94" s="65" t="inlineStr">
         <is>
@@ -8780,10 +8884,9 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B95" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
-        </is>
+      <c r="B95" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C95" s="65" t="inlineStr">
         <is>
@@ -8817,10 +8920,9 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B96" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
-        </is>
+      <c r="B96" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
+        <v/>
       </c>
       <c r="C96" s="65" t="inlineStr">
         <is>
@@ -8854,10 +8956,9 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B97" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
-        </is>
+      <c r="B97" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg")</f>
+        <v/>
       </c>
       <c r="C97" s="65" t="inlineStr">
         <is>
@@ -8891,10 +8992,9 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B98" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
-        </is>
+      <c r="B98" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C98" s="65" t="inlineStr">
         <is>
@@ -8928,10 +9028,9 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B99" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
-        </is>
+      <c r="B99" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C99" s="65" t="inlineStr">
         <is>
@@ -8965,10 +9064,9 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B100" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
-        </is>
+      <c r="B100" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C100" s="65" t="inlineStr">
         <is>
@@ -9002,10 +9100,9 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B101" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
-        </is>
+      <c r="B101" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C101" s="65" t="inlineStr">
         <is>
@@ -9039,10 +9136,9 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B102" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
-        </is>
+      <c r="B102" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml")</f>
+        <v/>
       </c>
       <c r="C102" s="65" t="inlineStr">
         <is>
@@ -9076,10 +9172,9 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B103" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
-        </is>
+      <c r="B103" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml")</f>
+        <v/>
       </c>
       <c r="C103" s="65" t="inlineStr">
         <is>
@@ -9113,10 +9208,9 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B104" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
-        </is>
+      <c r="B104" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml")</f>
+        <v/>
       </c>
       <c r="C104" s="65" t="inlineStr">
         <is>
@@ -9150,10 +9244,9 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B105" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
-        </is>
+      <c r="B105" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml")</f>
+        <v/>
       </c>
       <c r="C105" s="65" t="inlineStr">
         <is>
@@ -9232,10 +9325,9 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B109" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
-        </is>
+      <c r="B109" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
+        <v/>
       </c>
       <c r="C109" s="65" t="inlineStr">
         <is>
@@ -9269,10 +9361,9 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B110" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
-        </is>
+      <c r="B110" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
+        <v/>
       </c>
       <c r="C110" s="65" t="inlineStr">
         <is>
@@ -9306,10 +9397,9 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B111" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
-        </is>
+      <c r="B111" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg")</f>
+        <v/>
       </c>
       <c r="C111" s="65" t="inlineStr">
         <is>
@@ -9343,10 +9433,9 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B112" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
+      <c r="B112" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
       </c>
       <c r="C112" s="65" t="inlineStr">
         <is>
@@ -9380,10 +9469,9 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B113" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
-        </is>
+      <c r="B113" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg")</f>
+        <v/>
       </c>
       <c r="C113" s="65" t="inlineStr">
         <is>
@@ -9417,10 +9505,9 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B114" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
-        </is>
+      <c r="B114" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
+        <v/>
       </c>
       <c r="C114" s="65" t="inlineStr">
         <is>
@@ -9454,10 +9541,9 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B115" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
-        </is>
+      <c r="B115" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg")</f>
+        <v/>
       </c>
       <c r="C115" s="65" t="inlineStr">
         <is>
@@ -9491,10 +9577,9 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B116" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
-        </is>
+      <c r="B116" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg")</f>
+        <v/>
       </c>
       <c r="C116" s="65" t="inlineStr">
         <is>
@@ -9528,10 +9613,9 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B117" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
-        </is>
+      <c r="B117" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg")</f>
+        <v/>
       </c>
       <c r="C117" s="65" t="inlineStr">
         <is>
@@ -9565,10 +9649,9 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B118" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
-        </is>
+      <c r="B118" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg")</f>
+        <v/>
       </c>
       <c r="C118" s="65" t="inlineStr">
         <is>
@@ -9602,10 +9685,9 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B119" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
-        </is>
+      <c r="B119" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg")</f>
+        <v/>
       </c>
       <c r="C119" s="65" t="inlineStr">
         <is>
@@ -9639,10 +9721,9 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B120" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
-        </is>
+      <c r="B120" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx")</f>
+        <v/>
       </c>
       <c r="C120" s="65" t="inlineStr">
         <is>
@@ -9721,10 +9802,9 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B124" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
-        </is>
+      <c r="B124" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
       </c>
       <c r="C124" s="65" t="inlineStr">
         <is>
@@ -9764,10 +9844,9 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B125" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
-        </is>
+      <c r="B125" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
       </c>
       <c r="C125" s="65" t="inlineStr">
         <is>
@@ -9807,10 +9886,9 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B126" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
-        </is>
+      <c r="B126" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
       </c>
       <c r="C126" s="65" t="inlineStr">
         <is>
@@ -9850,10 +9928,9 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B127" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
-        </is>
+      <c r="B127" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx","\","/"),"02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx")</f>
+        <v/>
       </c>
       <c r="C127" s="65" t="inlineStr">
         <is>
@@ -9893,10 +9970,9 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B128" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
-        </is>
+      <c r="B128" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
       </c>
       <c r="C128" s="65" t="inlineStr">
         <is>
@@ -9936,10 +10012,9 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B129" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
-        </is>
+      <c r="B129" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
+        <v/>
       </c>
       <c r="C129" s="65" t="inlineStr">
         <is>
@@ -9976,10 +10051,9 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B130" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
-        </is>
+      <c r="B130" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C130" s="65" t="inlineStr">
         <is>
@@ -10016,10 +10090,9 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B131" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
-        </is>
+      <c r="B131" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
+        <v/>
       </c>
       <c r="C131" s="65" t="inlineStr">
         <is>
@@ -10061,10 +10134,9 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B132" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
-        </is>
+      <c r="B132" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C132" s="65" t="inlineStr">
         <is>
@@ -10101,10 +10173,9 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B133" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
-        </is>
+      <c r="B133" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
+        <v/>
       </c>
       <c r="C133" s="65" t="inlineStr">
         <is>
@@ -10141,10 +10212,9 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B134" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
-        </is>
+      <c r="B134" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg")</f>
+        <v/>
       </c>
       <c r="C134" s="65" t="inlineStr">
         <is>
@@ -10181,10 +10251,9 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B135" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
-        </is>
+      <c r="B135" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C135" s="65" t="inlineStr">
         <is>
@@ -10221,10 +10290,9 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B136" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
-        </is>
+      <c r="B136" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C136" s="65" t="inlineStr">
         <is>
@@ -10261,10 +10329,9 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B137" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
-        </is>
+      <c r="B137" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C137" s="65" t="inlineStr">
         <is>
@@ -10301,10 +10368,9 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B138" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
-        </is>
+      <c r="B138" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg")</f>
+        <v/>
       </c>
       <c r="C138" s="65" t="inlineStr">
         <is>
@@ -10341,10 +10407,9 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B139" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
-        </is>
+      <c r="B139" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml")</f>
+        <v/>
       </c>
       <c r="C139" s="65" t="inlineStr">
         <is>
@@ -10381,10 +10446,9 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B140" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
-        </is>
+      <c r="B140" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml")</f>
+        <v/>
       </c>
       <c r="C140" s="65" t="inlineStr">
         <is>
@@ -10421,10 +10485,9 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B141" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
-        </is>
+      <c r="B141" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml")</f>
+        <v/>
       </c>
       <c r="C141" s="65" t="inlineStr">
         <is>
@@ -10461,10 +10524,9 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B142" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
-        </is>
+      <c r="B142" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml")</f>
+        <v/>
       </c>
       <c r="C142" s="65" t="inlineStr">
         <is>
@@ -10498,10 +10560,9 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B143" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png</t>
-        </is>
+      <c r="B143" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png")</f>
+        <v/>
       </c>
       <c r="C143" s="65" t="inlineStr">
         <is>
@@ -10537,10 +10598,9 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B144" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
-        </is>
+      <c r="B144" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
+        <v/>
       </c>
       <c r="C144" s="65" t="inlineStr">
         <is>
@@ -10579,10 +10639,9 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B145" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
-        </is>
+      <c r="B145" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg")</f>
+        <v/>
       </c>
       <c r="C145" s="65" t="inlineStr">
         <is>
@@ -10618,10 +10677,9 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B146" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
+      <c r="B146" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
       </c>
       <c r="C146" s="65" t="inlineStr">
         <is>
@@ -10666,10 +10724,9 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B147" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
-        </is>
+      <c r="B147" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg")</f>
+        <v/>
       </c>
       <c r="C147" s="65" t="inlineStr">
         <is>
@@ -10708,10 +10765,9 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B148" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
-        </is>
+      <c r="B148" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
+        <v/>
       </c>
       <c r="C148" s="65" t="inlineStr">
         <is>
@@ -10746,10 +10802,9 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B149" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
-        </is>
+      <c r="B149" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg")</f>
+        <v/>
       </c>
       <c r="C149" s="65" t="inlineStr">
         <is>
@@ -10783,10 +10838,9 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B150" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
-        </is>
+      <c r="B150" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg")</f>
+        <v/>
       </c>
       <c r="C150" s="65" t="inlineStr">
         <is>
@@ -10821,10 +10875,9 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B151" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
-        </is>
+      <c r="B151" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg")</f>
+        <v/>
       </c>
       <c r="C151" s="65" t="inlineStr">
         <is>
@@ -10864,10 +10917,9 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B152" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
-        </is>
+      <c r="B152" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg")</f>
+        <v/>
       </c>
       <c r="C152" s="65" t="inlineStr">
         <is>
@@ -10901,10 +10953,9 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B153" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
-        </is>
+      <c r="B153" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg")</f>
+        <v/>
       </c>
       <c r="C153" s="65" t="inlineStr">
         <is>
@@ -10938,10 +10989,9 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B154" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
-        </is>
+      <c r="B154" s="64">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx")</f>
+        <v/>
       </c>
       <c r="C154" s="65" t="inlineStr">
         <is>
@@ -11821,7 +11871,6 @@
     <hyperlink ref="B18" location="'Application Attribute Testing'!A122" display="Evidence reference table – evidence number → attribute tests"/>
     <hyperlink ref="B19" location="'Application Attribute Testing'!A156" display="Conclusion – all applications in scope (PASS) with evidence references"/>
     <hyperlink ref="A23" location="'Application Attribute Testing'!A109" display="MA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" tooltip="Open evidence file" r:id="rId1"/>
     <hyperlink ref="H23" location="'Application Attribute Testing'!A109" display="MA01"/>
     <hyperlink ref="I23" location="'Application Attribute Testing'!A110" display="E01"/>
     <hyperlink ref="J23" location="'Application Attribute Testing'!A111" display="E02"/>
@@ -11829,7 +11878,6 @@
     <hyperlink ref="L23" location="'Application Attribute Testing'!A113" display="E04"/>
     <hyperlink ref="M23" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A27" location="'Application Attribute Testing'!A110" display="E01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" tooltip="Open evidence file" r:id="rId2"/>
     <hyperlink ref="H27" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I27" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J27" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11840,7 +11888,6 @@
     <hyperlink ref="O27" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="P27" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A32" location="'Application Attribute Testing'!A112" display="E03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" tooltip="Open evidence file" r:id="rId3"/>
     <hyperlink ref="H32" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I32" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J32" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11851,7 +11898,6 @@
     <hyperlink ref="O32" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="P32" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A36" location="'Application Attribute Testing'!A112" display="E03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" tooltip="Open evidence file" r:id="rId4"/>
     <hyperlink ref="H36" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I36" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J36" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11863,7 +11909,6 @@
     <hyperlink ref="P36" location="'Application Attribute Testing'!A116" display="E08"/>
     <hyperlink ref="Q36" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A40" location="'Application Attribute Testing'!A112" display="E03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" tooltip="Open evidence file" r:id="rId5"/>
     <hyperlink ref="H40" location="'Application Attribute Testing'!A89" display="BLA06"/>
     <hyperlink ref="I40" location="'Application Attribute Testing'!A93" display="DMA01"/>
     <hyperlink ref="J40" location="'Application Attribute Testing'!A94" display="DMA02"/>
@@ -11881,7 +11926,6 @@
     <hyperlink ref="V40" location="'Application Attribute Testing'!A113" display="E04"/>
     <hyperlink ref="W40" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A44" location="'Application Attribute Testing'!A112" display="E03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" tooltip="Open evidence file" r:id="rId6"/>
     <hyperlink ref="H44" location="'Application Attribute Testing'!A89" display="BLA06"/>
     <hyperlink ref="I44" location="'Application Attribute Testing'!A93" display="DMA01"/>
     <hyperlink ref="J44" location="'Application Attribute Testing'!A94" display="DMA02"/>
@@ -11899,7 +11943,6 @@
     <hyperlink ref="V44" location="'Application Attribute Testing'!A113" display="E04"/>
     <hyperlink ref="W44" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A48" location="'Application Attribute Testing'!A112" display="E03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" tooltip="Open evidence file" r:id="rId7"/>
     <hyperlink ref="H48" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I48" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J48" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11908,7 +11951,6 @@
     <hyperlink ref="M48" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="N48" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A52" location="'Application Attribute Testing'!A89" display="BLA06"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" tooltip="Open evidence file" r:id="rId8"/>
     <hyperlink ref="H52" location="'Application Attribute Testing'!A89" display="BLA06"/>
     <hyperlink ref="I52" location="'Application Attribute Testing'!A93" display="DMA01"/>
     <hyperlink ref="J52" location="'Application Attribute Testing'!A94" display="DMA02"/>
@@ -11924,15 +11966,10 @@
     <hyperlink ref="T52" location="'Application Attribute Testing'!A104" display="DMA12"/>
     <hyperlink ref="U52" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A53" location="'Application Attribute Testing'!A93" display="DMA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" tooltip="Open evidence file" r:id="rId9"/>
     <hyperlink ref="A54" location="'Application Attribute Testing'!A94" display="DMA02"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" tooltip="Open evidence file" r:id="rId10"/>
     <hyperlink ref="A55" location="'Application Attribute Testing'!A95" display="DMA03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" tooltip="Open evidence file" r:id="rId11"/>
     <hyperlink ref="A56" location="'Application Attribute Testing'!A96" display="DMA04"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" tooltip="Open evidence file" r:id="rId12"/>
     <hyperlink ref="A60" location="'Application Attribute Testing'!A112" display="E03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" tooltip="Open evidence file" r:id="rId13"/>
     <hyperlink ref="H60" location="'Application Attribute Testing'!A109" display="MA01"/>
     <hyperlink ref="I60" location="'Application Attribute Testing'!A110" display="E01"/>
     <hyperlink ref="J60" location="'Application Attribute Testing'!A111" display="E02"/>
@@ -11940,7 +11977,6 @@
     <hyperlink ref="L60" location="'Application Attribute Testing'!A113" display="E04"/>
     <hyperlink ref="M60" location="'Application Attribute Testing'!A120" display="E16b"/>
     <hyperlink ref="A64" location="'Application Attribute Testing'!A110" display="E01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" tooltip="Open evidence file" r:id="rId14"/>
     <hyperlink ref="H64" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I64" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J64" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11950,7 +11986,6 @@
     <hyperlink ref="N64" location="'Application Attribute Testing'!A110" display="E01"/>
     <hyperlink ref="O64" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="A68" location="'Application Attribute Testing'!A114" display="E05"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" tooltip="Open evidence file" r:id="rId15"/>
     <hyperlink ref="H68" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I68" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J68" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11963,7 +11998,6 @@
     <hyperlink ref="Q68" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="R68" location="'Application Attribute Testing'!A118" display="E10"/>
     <hyperlink ref="A72" location="'Application Attribute Testing'!A109" display="MA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" tooltip="Open evidence file" r:id="rId16"/>
     <hyperlink ref="H72" location="'Application Attribute Testing'!A94" display="DMA02"/>
     <hyperlink ref="I72" location="'Application Attribute Testing'!A109" display="MA01"/>
     <hyperlink ref="J72" location="'Application Attribute Testing'!A110" display="E01"/>
@@ -11971,7 +12005,6 @@
     <hyperlink ref="L72" location="'Application Attribute Testing'!A114" display="E05"/>
     <hyperlink ref="M72" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A76" location="'Application Attribute Testing'!A89" display="BLA06"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" tooltip="Open evidence file" r:id="rId17"/>
     <hyperlink ref="H76" location="'Application Attribute Testing'!A84" display="BLA01"/>
     <hyperlink ref="I76" location="'Application Attribute Testing'!A85" display="BLA02"/>
     <hyperlink ref="J76" location="'Application Attribute Testing'!A86" display="BLA03"/>
@@ -11993,106 +12026,40 @@
     <hyperlink ref="Z76" location="'Application Attribute Testing'!A112" display="E03"/>
     <hyperlink ref="AA76" location="'Application Attribute Testing'!A117" display="E09"/>
     <hyperlink ref="A77" location="'Application Attribute Testing'!A93" display="DMA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" tooltip="Open evidence file" r:id="rId18"/>
     <hyperlink ref="A78" location="'Application Attribute Testing'!A94" display="DMA02"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" tooltip="Open evidence file" r:id="rId19"/>
     <hyperlink ref="A79" location="'Application Attribute Testing'!A95" display="DMA03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" tooltip="Open evidence file" r:id="rId20"/>
     <hyperlink ref="A80" location="'Application Attribute Testing'!A96" display="DMA04"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" tooltip="Open evidence file" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" tooltip="Open evidence file" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B85" tooltip="Open evidence file" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" tooltip="Open evidence file" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" tooltip="Open evidence file" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" tooltip="Open evidence file" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" tooltip="Open evidence file" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" tooltip="Open evidence file" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" tooltip="Open evidence file" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" tooltip="Open evidence file" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" tooltip="Open evidence file" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" tooltip="Open evidence file" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" tooltip="Open evidence file" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" tooltip="Open evidence file" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" tooltip="Open evidence file" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" tooltip="Open evidence file" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" tooltip="Open evidence file" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" tooltip="Open evidence file" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" tooltip="Open evidence file" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B105" tooltip="Open evidence file" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" tooltip="Open evidence file" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" tooltip="Open evidence file" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" tooltip="Open evidence file" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" tooltip="Open evidence file" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" tooltip="Open evidence file" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" tooltip="Open evidence file" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" tooltip="Open evidence file" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" tooltip="Open evidence file" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B117" tooltip="Open evidence file" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" tooltip="Open evidence file" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B119" tooltip="Open evidence file" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" tooltip="Open evidence file" r:id="rId52"/>
     <hyperlink ref="A124" location="'Application Attribute Testing'!A84" display="BLA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" tooltip="Open evidence file" r:id="rId53"/>
     <hyperlink ref="A125" location="'Application Attribute Testing'!A85" display="BLA02"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" tooltip="Open evidence file" r:id="rId54"/>
     <hyperlink ref="A126" location="'Application Attribute Testing'!A86" display="BLA03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" tooltip="Open evidence file" r:id="rId55"/>
     <hyperlink ref="A127" location="'Application Attribute Testing'!A87" display="BLA04"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" tooltip="Open evidence file" r:id="rId56"/>
     <hyperlink ref="A128" location="'Application Attribute Testing'!A88" display="BLA05"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" tooltip="Open evidence file" r:id="rId57"/>
     <hyperlink ref="A129" location="'Application Attribute Testing'!A89" display="BLA06"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" tooltip="Open evidence file" r:id="rId58"/>
     <hyperlink ref="A130" location="'Application Attribute Testing'!A93" display="DMA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" tooltip="Open evidence file" r:id="rId59"/>
     <hyperlink ref="A131" location="'Application Attribute Testing'!A94" display="DMA02"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" tooltip="Open evidence file" r:id="rId60"/>
     <hyperlink ref="A132" location="'Application Attribute Testing'!A95" display="DMA03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B132" tooltip="Open evidence file" r:id="rId61"/>
     <hyperlink ref="A133" location="'Application Attribute Testing'!A96" display="DMA04"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B133" tooltip="Open evidence file" r:id="rId62"/>
     <hyperlink ref="A134" location="'Application Attribute Testing'!A97" display="DMA05"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B134" tooltip="Open evidence file" r:id="rId63"/>
     <hyperlink ref="A135" location="'Application Attribute Testing'!A98" display="DMA06"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B135" tooltip="Open evidence file" r:id="rId64"/>
     <hyperlink ref="A136" location="'Application Attribute Testing'!A99" display="DMA07"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B136" tooltip="Open evidence file" r:id="rId65"/>
     <hyperlink ref="A137" location="'Application Attribute Testing'!A100" display="DMA08"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B137" tooltip="Open evidence file" r:id="rId66"/>
     <hyperlink ref="A138" location="'Application Attribute Testing'!A101" display="DMA09"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" tooltip="Open evidence file" r:id="rId67"/>
     <hyperlink ref="A139" location="'Application Attribute Testing'!A102" display="DMA10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" tooltip="Open evidence file" r:id="rId68"/>
     <hyperlink ref="A140" location="'Application Attribute Testing'!A103" display="DMA11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" tooltip="Open evidence file" r:id="rId69"/>
     <hyperlink ref="A141" location="'Application Attribute Testing'!A104" display="DMA12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B141" tooltip="Open evidence file" r:id="rId70"/>
     <hyperlink ref="A142" location="'Application Attribute Testing'!A105" display="DMA13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B142" tooltip="Open evidence file" r:id="rId71"/>
     <hyperlink ref="A143" location="'Application Attribute Testing'!A109" display="MA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" tooltip="Open evidence file" r:id="rId72"/>
     <hyperlink ref="A144" location="'Application Attribute Testing'!A110" display="E01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" tooltip="Open evidence file" r:id="rId73"/>
     <hyperlink ref="A145" location="'Application Attribute Testing'!A111" display="E02"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" tooltip="Open evidence file" r:id="rId74"/>
     <hyperlink ref="A146" location="'Application Attribute Testing'!A112" display="E03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B146" tooltip="Open evidence file" r:id="rId75"/>
     <hyperlink ref="A147" location="'Application Attribute Testing'!A113" display="E04"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" tooltip="Open evidence file" r:id="rId76"/>
     <hyperlink ref="A148" location="'Application Attribute Testing'!A114" display="E05"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" tooltip="Open evidence file" r:id="rId77"/>
     <hyperlink ref="A149" location="'Application Attribute Testing'!A115" display="E07"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" tooltip="Open evidence file" r:id="rId78"/>
     <hyperlink ref="A150" location="'Application Attribute Testing'!A116" display="E08"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B150" tooltip="Open evidence file" r:id="rId79"/>
     <hyperlink ref="A151" location="'Application Attribute Testing'!A117" display="E09"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B151" tooltip="Open evidence file" r:id="rId80"/>
     <hyperlink ref="A152" location="'Application Attribute Testing'!A118" display="E10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B152" tooltip="Open evidence file" r:id="rId81"/>
     <hyperlink ref="A153" location="'Application Attribute Testing'!A119" display="E13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B153" tooltip="Open evidence file" r:id="rId82"/>
     <hyperlink ref="A154" location="'Application Attribute Testing'!A120" display="E16b"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B154" tooltip="Open evidence file" r:id="rId83"/>
     <hyperlink ref="A158" location="'Application Attribute Testing-1'!A3" display="1822"/>
     <hyperlink ref="B158" location="'Application Attribute Testing-1'!A3" display="ACH Express"/>
     <hyperlink ref="A159" location="'Application Attribute Testing-1'!A4" display="1867"/>
@@ -13999,15 +13966,13 @@
           <t>MA01</t>
         </is>
       </c>
-      <c r="B3" s="92" t="inlineStr">
-        <is>
-          <t>MA01_BSI In-Scope Applications-2026.png</t>
-        </is>
-      </c>
-      <c r="C3" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications</t>
-        </is>
+      <c r="B3" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png","\","/"),"01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png"),"MA01_BSI In-Scope Applications-2026.png")</f>
+        <v/>
+      </c>
+      <c r="C3" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("01_Management_Attestation_In-Scope_Applications","\","/"),"01_Management_Attestation_In-Scope_Applications"),"BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications")</f>
+        <v/>
       </c>
       <c r="D3" s="35" t="inlineStr">
         <is>
@@ -14053,15 +14018,13 @@
           <t>BLA01</t>
         </is>
       </c>
-      <c r="B4" s="92" t="inlineStr">
-        <is>
-          <t>BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
-        </is>
-      </c>
-      <c r="C4" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
-        </is>
+      <c r="B4" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf"),"BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
+      </c>
+      <c r="C4" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
+        <v/>
       </c>
       <c r="D4" s="35" t="inlineStr">
         <is>
@@ -14107,15 +14070,13 @@
           <t>BLA02</t>
         </is>
       </c>
-      <c r="B5" s="92" t="inlineStr">
-        <is>
-          <t>BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
-        </is>
-      </c>
-      <c r="C5" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
-        </is>
+      <c r="B5" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf"),"BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
+      </c>
+      <c r="C5" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
+        <v/>
       </c>
       <c r="D5" s="35" t="inlineStr">
         <is>
@@ -14161,15 +14122,13 @@
           <t>BLA03</t>
         </is>
       </c>
-      <c r="B6" s="92" t="inlineStr">
-        <is>
-          <t>BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
-        </is>
-      </c>
-      <c r="C6" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
-        </is>
+      <c r="B6" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf"),"BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
+      </c>
+      <c r="C6" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
+        <v/>
       </c>
       <c r="D6" s="35" t="inlineStr">
         <is>
@@ -14215,15 +14174,13 @@
           <t>BLA04</t>
         </is>
       </c>
-      <c r="B7" s="92" t="inlineStr">
-        <is>
-          <t>BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
-        </is>
-      </c>
-      <c r="C7" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
-        </is>
+      <c r="B7" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx","\","/"),"02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx"),"BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx")</f>
+        <v/>
+      </c>
+      <c r="C7" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
+        <v/>
       </c>
       <c r="D7" s="35" t="inlineStr">
         <is>
@@ -14269,15 +14226,13 @@
           <t>BLA05</t>
         </is>
       </c>
-      <c r="B8" s="92" t="inlineStr">
-        <is>
-          <t>BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
-        </is>
-      </c>
-      <c r="C8" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
-        </is>
+      <c r="B8" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf","\","/"),"02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf"),"BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf")</f>
+        <v/>
+      </c>
+      <c r="C8" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
+        <v/>
       </c>
       <c r="D8" s="35" t="inlineStr">
         <is>
@@ -14323,15 +14278,13 @@
           <t>BLA06</t>
         </is>
       </c>
-      <c r="B9" s="92" t="inlineStr">
-        <is>
-          <t>BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
-        </is>
-      </c>
-      <c r="C9" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
-        </is>
+      <c r="B9" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg","\","/"),"02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg"),"BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C9" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("02_Business_Line_Approval_Results_Email","\","/"),"02_Business_Line_Approval_Results_Email"),"BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email")</f>
+        <v/>
       </c>
       <c r="D9" s="35" t="inlineStr">
         <is>
@@ -14377,15 +14330,13 @@
           <t>DMA01</t>
         </is>
       </c>
-      <c r="B10" s="92" t="inlineStr">
-        <is>
-          <t>DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
-        </is>
-      </c>
-      <c r="C10" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B10" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg"),"DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C10" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D10" s="35" t="inlineStr">
         <is>
@@ -14431,15 +14382,13 @@
           <t>DMA02</t>
         </is>
       </c>
-      <c r="B11" s="92" t="inlineStr">
-        <is>
-          <t>DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
-        </is>
-      </c>
-      <c r="C11" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B11" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg"),"DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C11" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D11" s="35" t="inlineStr">
         <is>
@@ -14485,15 +14434,13 @@
           <t>DMA03</t>
         </is>
       </c>
-      <c r="B12" s="92" t="inlineStr">
-        <is>
-          <t>DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
-        </is>
-      </c>
-      <c r="C12" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B12" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg"),"DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C12" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D12" s="35" t="inlineStr">
         <is>
@@ -14539,15 +14486,13 @@
           <t>DMA04</t>
         </is>
       </c>
-      <c r="B13" s="92" t="inlineStr">
-        <is>
-          <t>DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
-        </is>
-      </c>
-      <c r="C13" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B13" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg"),"DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C13" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D13" s="35" t="inlineStr">
         <is>
@@ -14593,15 +14538,13 @@
           <t>DMA05</t>
         </is>
       </c>
-      <c r="B14" s="92" t="inlineStr">
-        <is>
-          <t>DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
-        </is>
-      </c>
-      <c r="C14" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B14" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg"),"DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C14" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D14" s="35" t="inlineStr">
         <is>
@@ -14647,15 +14590,13 @@
           <t>DMA06</t>
         </is>
       </c>
-      <c r="B15" s="92" t="inlineStr">
-        <is>
-          <t>DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
-        </is>
-      </c>
-      <c r="C15" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B15" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg"),"DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C15" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D15" s="35" t="inlineStr">
         <is>
@@ -14701,15 +14642,13 @@
           <t>DMA07</t>
         </is>
       </c>
-      <c r="B16" s="92" t="inlineStr">
-        <is>
-          <t>DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
-        </is>
-      </c>
-      <c r="C16" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B16" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg"),"DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C16" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D16" s="35" t="inlineStr">
         <is>
@@ -14755,15 +14694,13 @@
           <t>DMA08</t>
         </is>
       </c>
-      <c r="B17" s="92" t="inlineStr">
-        <is>
-          <t>DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
-        </is>
-      </c>
-      <c r="C17" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B17" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg"),"DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C17" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D17" s="35" t="inlineStr">
         <is>
@@ -14809,15 +14746,13 @@
           <t>DMA09</t>
         </is>
       </c>
-      <c r="B18" s="92" t="inlineStr">
-        <is>
-          <t>DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
-        </is>
-      </c>
-      <c r="C18" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B18" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg"),"DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg")</f>
+        <v/>
+      </c>
+      <c r="C18" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D18" s="35" t="inlineStr">
         <is>
@@ -14863,15 +14798,13 @@
           <t>DMA10</t>
         </is>
       </c>
-      <c r="B19" s="92" t="inlineStr">
-        <is>
-          <t>DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
-        </is>
-      </c>
-      <c r="C19" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B19" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml"),"DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml")</f>
+        <v/>
+      </c>
+      <c r="C19" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D19" s="35" t="inlineStr">
         <is>
@@ -14917,15 +14850,13 @@
           <t>DMA11</t>
         </is>
       </c>
-      <c r="B20" s="92" t="inlineStr">
-        <is>
-          <t>DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
-        </is>
-      </c>
-      <c r="C20" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B20" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml"),"DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml")</f>
+        <v/>
+      </c>
+      <c r="C20" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D20" s="35" t="inlineStr">
         <is>
@@ -14971,15 +14902,13 @@
           <t>DMA12</t>
         </is>
       </c>
-      <c r="B21" s="92" t="inlineStr">
-        <is>
-          <t>DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
-        </is>
-      </c>
-      <c r="C21" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B21" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml"),"DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml")</f>
+        <v/>
+      </c>
+      <c r="C21" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D21" s="35" t="inlineStr">
         <is>
@@ -15025,15 +14954,13 @@
           <t>DMA13</t>
         </is>
       </c>
-      <c r="B22" s="92" t="inlineStr">
-        <is>
-          <t>DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
-        </is>
-      </c>
-      <c r="C22" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
-        </is>
+      <c r="B22" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml","\","/"),"03_DIV_Manager_Attestation_Email_Approvals\DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml"),"DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml")</f>
+        <v/>
+      </c>
+      <c r="C22" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("03_DIV_Manager_Attestation_Email_Approvals","\","/"),"03_DIV_Manager_Attestation_Email_Approvals"),"BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals")</f>
+        <v/>
       </c>
       <c r="D22" s="35" t="inlineStr">
         <is>
@@ -15079,15 +15006,13 @@
           <t>E01</t>
         </is>
       </c>
-      <c r="B23" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
-        </is>
-      </c>
-      <c r="C23" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B23" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx"),"BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx")</f>
+        <v/>
+      </c>
+      <c r="C23" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D23" s="35" t="inlineStr">
         <is>
@@ -15133,15 +15058,13 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B24" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
-        </is>
-      </c>
-      <c r="C24" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B24" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg"),"BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg")</f>
+        <v/>
+      </c>
+      <c r="C24" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D24" s="35" t="inlineStr">
         <is>
@@ -15187,15 +15110,13 @@
           <t>E03</t>
         </is>
       </c>
-      <c r="B25" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
-        </is>
-      </c>
-      <c r="C25" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B25" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls"),"BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls")</f>
+        <v/>
+      </c>
+      <c r="C25" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D25" s="35" t="inlineStr">
         <is>
@@ -15241,15 +15162,13 @@
           <t>E04</t>
         </is>
       </c>
-      <c r="B26" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
-        </is>
-      </c>
-      <c r="C26" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B26" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg"),"BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg")</f>
+        <v/>
+      </c>
+      <c r="C26" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D26" s="35" t="inlineStr">
         <is>
@@ -15295,15 +15214,13 @@
           <t>E05</t>
         </is>
       </c>
-      <c r="B27" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
-        </is>
-      </c>
-      <c r="C27" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B27" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg"),"BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg")</f>
+        <v/>
+      </c>
+      <c r="C27" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D27" s="35" t="inlineStr">
         <is>
@@ -15349,15 +15266,13 @@
           <t>E07</t>
         </is>
       </c>
-      <c r="B28" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
-        </is>
-      </c>
-      <c r="C28" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B28" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg"),"BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg")</f>
+        <v/>
+      </c>
+      <c r="C28" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D28" s="35" t="inlineStr">
         <is>
@@ -15403,15 +15318,13 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B29" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
-        </is>
-      </c>
-      <c r="C29" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B29" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg"),"BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg")</f>
+        <v/>
+      </c>
+      <c r="C29" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D29" s="35" t="inlineStr">
         <is>
@@ -15457,15 +15370,13 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B30" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
-        </is>
-      </c>
-      <c r="C30" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B30" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg"),"BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg")</f>
+        <v/>
+      </c>
+      <c r="C30" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D30" s="35" t="inlineStr">
         <is>
@@ -15511,15 +15422,13 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="B31" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
-        </is>
-      </c>
-      <c r="C31" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B31" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg"),"BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg")</f>
+        <v/>
+      </c>
+      <c r="C31" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D31" s="35" t="inlineStr">
         <is>
@@ -15565,15 +15474,13 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B32" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
-        </is>
-      </c>
-      <c r="C32" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B32" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg"),"BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg")</f>
+        <v/>
+      </c>
+      <c r="C32" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D32" s="35" t="inlineStr">
         <is>
@@ -15619,15 +15526,13 @@
           <t>E16b</t>
         </is>
       </c>
-      <c r="B33" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
-        </is>
-      </c>
-      <c r="C33" s="92" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
-        </is>
+      <c r="B33" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx"),"BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx")</f>
+        <v/>
+      </c>
+      <c r="C33" s="92">
+        <f>HYPERLINK(EvidenceRoot&amp;IF(LEFT(EvidenceRoot,4)="http",SUBSTITUTE("04_Data_Integrity_and_Email_Testing_Evidence","\","/"),"04_Data_Integrity_and_Email_Testing_Evidence"),"BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence")</f>
+        <v/>
       </c>
       <c r="D33" s="35" t="inlineStr">
         <is>
@@ -17373,98 +17278,36 @@
   <autoFilter ref="A2:K33"/>
   <hyperlinks>
     <hyperlink ref="A3" location="'Application Attribute Testing'!A109" display="MA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" tooltip="Open evidence file" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" tooltip="Open evidence folder" r:id="rId2"/>
     <hyperlink ref="A4" location="'Application Attribute Testing'!A84" display="BLA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" tooltip="Open evidence file" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" tooltip="Open evidence folder" r:id="rId4"/>
     <hyperlink ref="A5" location="'Application Attribute Testing'!A85" display="BLA02"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" tooltip="Open evidence file" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" tooltip="Open evidence folder" r:id="rId6"/>
     <hyperlink ref="A6" location="'Application Attribute Testing'!A86" display="BLA03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" tooltip="Open evidence file" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" tooltip="Open evidence folder" r:id="rId8"/>
     <hyperlink ref="A7" location="'Application Attribute Testing'!A87" display="BLA04"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" tooltip="Open evidence file" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" tooltip="Open evidence folder" r:id="rId10"/>
     <hyperlink ref="A8" location="'Application Attribute Testing'!A88" display="BLA05"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" tooltip="Open evidence file" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" tooltip="Open evidence folder" r:id="rId12"/>
     <hyperlink ref="A9" location="'Application Attribute Testing'!A89" display="BLA06"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" tooltip="Open evidence file" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" tooltip="Open evidence folder" r:id="rId14"/>
     <hyperlink ref="A10" location="'Application Attribute Testing'!A93" display="DMA01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" tooltip="Open evidence file" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" tooltip="Open evidence folder" r:id="rId16"/>
     <hyperlink ref="A11" location="'Application Attribute Testing'!A94" display="DMA02"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" tooltip="Open evidence file" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" tooltip="Open evidence folder" r:id="rId18"/>
     <hyperlink ref="A12" location="'Application Attribute Testing'!A95" display="DMA03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" tooltip="Open evidence file" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" tooltip="Open evidence folder" r:id="rId20"/>
     <hyperlink ref="A13" location="'Application Attribute Testing'!A96" display="DMA04"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" tooltip="Open evidence file" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" tooltip="Open evidence folder" r:id="rId22"/>
     <hyperlink ref="A14" location="'Application Attribute Testing'!A97" display="DMA05"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" tooltip="Open evidence file" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" tooltip="Open evidence folder" r:id="rId24"/>
     <hyperlink ref="A15" location="'Application Attribute Testing'!A98" display="DMA06"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" tooltip="Open evidence file" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" tooltip="Open evidence folder" r:id="rId26"/>
     <hyperlink ref="A16" location="'Application Attribute Testing'!A99" display="DMA07"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" tooltip="Open evidence file" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" tooltip="Open evidence folder" r:id="rId28"/>
     <hyperlink ref="A17" location="'Application Attribute Testing'!A100" display="DMA08"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" tooltip="Open evidence file" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" tooltip="Open evidence folder" r:id="rId30"/>
     <hyperlink ref="A18" location="'Application Attribute Testing'!A101" display="DMA09"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" tooltip="Open evidence file" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" tooltip="Open evidence folder" r:id="rId32"/>
     <hyperlink ref="A19" location="'Application Attribute Testing'!A102" display="DMA10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" tooltip="Open evidence file" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" tooltip="Open evidence folder" r:id="rId34"/>
     <hyperlink ref="A20" location="'Application Attribute Testing'!A103" display="DMA11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" tooltip="Open evidence file" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" tooltip="Open evidence folder" r:id="rId36"/>
     <hyperlink ref="A21" location="'Application Attribute Testing'!A104" display="DMA12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" tooltip="Open evidence file" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" tooltip="Open evidence folder" r:id="rId38"/>
     <hyperlink ref="A22" location="'Application Attribute Testing'!A105" display="DMA13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" tooltip="Open evidence file" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" tooltip="Open evidence folder" r:id="rId40"/>
     <hyperlink ref="A23" location="'Application Attribute Testing'!A110" display="E01"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" tooltip="Open evidence file" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" tooltip="Open evidence folder" r:id="rId42"/>
     <hyperlink ref="A24" location="'Application Attribute Testing'!A111" display="E02"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" tooltip="Open evidence file" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" tooltip="Open evidence folder" r:id="rId44"/>
     <hyperlink ref="A25" location="'Application Attribute Testing'!A112" display="E03"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" tooltip="Open evidence file" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" tooltip="Open evidence folder" r:id="rId46"/>
     <hyperlink ref="A26" location="'Application Attribute Testing'!A113" display="E04"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" tooltip="Open evidence file" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" tooltip="Open evidence folder" r:id="rId48"/>
     <hyperlink ref="A27" location="'Application Attribute Testing'!A114" display="E05"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" tooltip="Open evidence file" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" tooltip="Open evidence folder" r:id="rId50"/>
     <hyperlink ref="A28" location="'Application Attribute Testing'!A115" display="E07"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" tooltip="Open evidence file" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" tooltip="Open evidence folder" r:id="rId52"/>
     <hyperlink ref="A29" location="'Application Attribute Testing'!A116" display="E08"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" tooltip="Open evidence file" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" tooltip="Open evidence folder" r:id="rId54"/>
     <hyperlink ref="A30" location="'Application Attribute Testing'!A117" display="E09"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" tooltip="Open evidence file" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" tooltip="Open evidence folder" r:id="rId56"/>
     <hyperlink ref="A31" location="'Application Attribute Testing'!A118" display="E10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" tooltip="Open evidence file" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" tooltip="Open evidence folder" r:id="rId58"/>
     <hyperlink ref="A32" location="'Application Attribute Testing'!A119" display="E13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" tooltip="Open evidence file" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" tooltip="Open evidence folder" r:id="rId60"/>
     <hyperlink ref="A33" location="'Application Attribute Testing'!A120" display="E16b"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" tooltip="Open evidence file" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" tooltip="Open evidence folder" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>